<commit_message>
added questions for cohort
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-BCS.xlsx
+++ b/baseline/data_processing_elements-BCS.xlsx
@@ -713,7 +713,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5.140625" customWidth="1" min="1" max="1"/>
-    <col hidden="1" min="2" max="2"/>
+    <col hidden="1" width="13" customWidth="1" min="2" max="2"/>
     <col width="22.7109375" customWidth="1" min="3" max="3"/>
     <col width="24.5703125" customWidth="1" min="4" max="4"/>
     <col width="4.140625" customWidth="1" min="7" max="8"/>
@@ -6003,7 +6003,11 @@
           <t>BA: confirm with the cohort, but usually if the participants were not required to be fasted, they are considered non-fasting</t>
         </is>
       </c>
-      <c r="AB40" s="2" t="n"/>
+      <c r="AB40" s="2" t="inlineStr">
+        <is>
+          <t>The data dictionary notes participants were not required to fast (nurse visits at any time of day). Was fasting status recorded per participant? If not, should all participants be coded non-fasting, or as unknown/NA?</t>
+        </is>
+      </c>
       <c r="AC40" s="2" t="inlineStr">
         <is>
           <t>I don't think we know what fasting state they were in,the dd states "Participants were not required to be in a fasted state as nurses made visits at any time in the day", so they could be in a fasting state or not so I think it should be NA/impossible</t>
@@ -8299,7 +8303,11 @@
 </t>
         </is>
       </c>
-      <c r="AB61" s="2" t="n"/>
+      <c r="AB61" s="2" t="inlineStr">
+        <is>
+          <t>To derive 'sleep difficulties', please clarify what B10TRBSLP (frequency of waking / trouble falling back asleep, last 4 weeks) captures, and whether B10TRBSLP / B10HSLEEP / B10FSLEEP together can identify participants with sleep difficulties.</t>
+        </is>
+      </c>
       <c r="AC61" s="2" t="n"/>
       <c r="AD61" s="2" t="n"/>
       <c r="AE61" s="2" t="n"/>
@@ -14496,7 +14504,11 @@
 - B10LNGDRC4 (1-10): BNF code subchapter</t>
         </is>
       </c>
-      <c r="AB113" s="2" t="n"/>
+      <c r="AB113" s="2" t="inlineStr">
+        <is>
+          <t>(1) Can all drugs under BNF section 2.12 (lipid-regulating drugs) be treated as lipid-lowering? (2) In medication variables such as B10MEDLNGW, should codes -9/-8/-1 be treated as missing (NA) or as 'no medication' (0)?</t>
+        </is>
+      </c>
       <c r="AC113" s="2" t="n"/>
       <c r="AD113" s="2" t="n"/>
       <c r="AE113" s="2" t="n"/>
@@ -15270,7 +15282,11 @@
           <t>if B10MEDLNGW %in% c(-9, -8, -1) is it NA or 0 refer to BCS mail question 2</t>
         </is>
       </c>
-      <c r="AB115" s="2" t="n"/>
+      <c r="AB115" s="2" t="inlineStr">
+        <is>
+          <t>In medication variables such as B10MEDLNGW, should codes -9/-8/-1 be treated as missing (NA) or as 'no medication' (0)?</t>
+        </is>
+      </c>
       <c r="AC115" s="2" t="n"/>
       <c r="AD115" s="2" t="n"/>
       <c r="AE115" s="2" t="n"/>

</xml_diff>

<commit_message>
Corrections after validation of harmo outputs
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-BCS.xlsx
+++ b/baseline/data_processing_elements-BCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9BBC454-598C-4D34-ABEB-55A03C5E1E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E547C0-2627-4353-856E-DD00455C7286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="1840" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2108" uniqueCount="995">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2109" uniqueCount="999">
   <si>
     <t>index</t>
   </si>
@@ -1654,11 +1654,6 @@
   </si>
   <si>
     <t>Friedewald equation was used</t>
-  </si>
-  <si>
-    <t>case_when(
-(B10CHOL &gt; 0) &amp; (B10HDL &gt; 0) &amp; (B10TRIG &gt; 0) ~ round(as.numeric(B10CHOL) - as.numeric(B10HDL) - (as.numeric(B10TRIG)/2.2), 2);
-ELSE ~ NA_real_)</t>
   </si>
   <si>
     <t>The number of decimals should be specified in the instructions.</t>
@@ -3886,17 +3881,7 @@
   </si>
   <si>
     <t>case_when(
-B10WAISTAV &gt; 0 ~ B10WAISTAV &gt; 0 ; 
-ELSE ~ NA_real_)</t>
-  </si>
-  <si>
-    <t>case_when(
 B10WAISTAV &gt; 0 ~ 2L ; 
-ELSE ~ NA_real_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10BFPC &gt; 0 ~ B10BFPC &gt; 0 ; 
 ELSE ~ NA_real_)</t>
   </si>
   <si>
@@ -3986,20 +3971,6 @@
   <si>
     <t>The study-specific variables were collected in categorical format with ranges of hours per week, so the midpoints of the ranges were used for calculations.
 Study-specific variables about TV programmes, videos, DVDs or Blu-ray, and watching programs or films on a computer were included.</t>
-  </si>
-  <si>
-    <t>The DataSchema variable was calculated using weighted values for study-specific variables about weekend and weekday behaviour.
-The study-specific variables were collected in categorical format with ranges of hours per week, so the midpoints of the ranges were used for calculations.
-Study-specific variables about TV programmes, videos, DVDs or Blu-ray, and watching programs or films on a computer were included.</t>
-  </si>
-  <si>
-    <t>The DataSchema variable was calculated using weighted values for study-specific variables about weekend and weekday behaviour.
-The study-specific variables were collected in categorical format with ranges of hours per week, so the midpoints of the ranges were used for calculations.</t>
-  </si>
-  <si>
-    <t>The DataSchema variable was calculated using weighted values for study-specific variables about weekend and weekday behaviour.
-The study-specific variables were collected in categorical format with ranges of hours per week, so the midpoints of the ranges were used for calculations.
-The study-specific variables were about reading at home, including in electronic format.</t>
   </si>
   <si>
     <t>Confirm that we don't have any variables besides B10ASITH Total sitting time over the day (hr/d) in main dataset (only from activpal)?</t>
@@ -4735,6 +4706,53 @@
   </si>
   <si>
     <t>Only one population.</t>
+  </si>
+  <si>
+    <t>Changed to code No.</t>
+  </si>
+  <si>
+    <t>recode(
+0=0;
+1=1;
+ELSE=NA)</t>
+  </si>
+  <si>
+    <t>Add condition "Leave missing when triglycerides exceed 4.5 mmol/L (400 mg/dL)."</t>
+  </si>
+  <si>
+    <t>case_when(
+ B10TRIG &gt; 4.5 ~  NA_real_ ; 
+(B10CHOL &gt; 0) &amp; (B10HDL &gt; 0) &amp; (B10TRIG &gt; 0) ~ round(as.numeric(B10CHOL) - as.numeric(B10HDL) - (as.numeric(B10TRIG)/2.2), 2);
+ELSE ~ NA_real_)</t>
+  </si>
+  <si>
+    <t>The DataSchema variable was calculated using weighted values for study-specific variables about weekend and weekday behaviour. Harmonized values are NA if either input variable is missing.
+The study-specific variables were collected in categorical format with ranges of hours per week, so the midpoints of the ranges were used for calculations.
+Study-specific variables about TV programmes, videos, DVDs or Blu-ray, and watching programs or films on a computer were included.</t>
+  </si>
+  <si>
+    <t>The DataSchema variable was calculated using weighted values for study-specific variables about weekend and weekday behaviour.  Harmonized values are NA if either input variable is missing.
+The study-specific variables were collected in categorical format with ranges of hours per week, so the midpoints of the ranges were used for calculations.</t>
+  </si>
+  <si>
+    <t>The DataSchema variable was calculated using weighted values for study-specific variables about weekend and weekday behaviour. Harmonized values are NA if either input variable is missing.
+The study-specific variables were collected in categorical format with ranges of hours per week, so the midpoints of the ranges were used for calculations.
+The study-specific variables were about reading at home, including in electronic format.</t>
+  </si>
+  <si>
+    <t>case_when(
+B10BFPC &gt; 0 ~ as.numeric(B10BFPC) ; 
+ELSE ~ NA_real_)</t>
+  </si>
+  <si>
+    <t>Variables like this should  be compatible if missing codes are changed.
+Changed to case_when.
+Already 1 decimal place.</t>
+  </si>
+  <si>
+    <t>case_when(
+B10WAISTAV &gt; 0 ~ as.numeric(B10WAISTAV) ; 
+ELSE ~ NA_real_)</t>
   </si>
 </sst>
 </file>
@@ -5551,7 +5569,7 @@
         <v>59</v>
       </c>
       <c r="AC4" s="22" t="s">
-        <v>994</v>
+        <v>988</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -5645,7 +5663,7 @@
         <v>78</v>
       </c>
       <c r="V6" s="22" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="W6" s="16" t="s">
         <v>44</v>
@@ -5769,13 +5787,13 @@
         <v>45</v>
       </c>
       <c r="Y8" s="24" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="Z8" s="24" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="AC8" s="18" t="s">
-        <v>970</v>
+        <v>964</v>
       </c>
     </row>
     <row r="9" spans="1:33" ht="180" x14ac:dyDescent="0.25">
@@ -5828,7 +5846,7 @@
         <v>116</v>
       </c>
       <c r="V9" s="22" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="W9" s="16" t="s">
         <v>44</v>
@@ -5840,19 +5858,19 @@
         <v>92</v>
       </c>
       <c r="Z9" s="14" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="AA9" s="18" t="s">
         <v>117</v>
       </c>
       <c r="AB9" s="23" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="AC9" s="22" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="AD9" s="23" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="10" spans="1:33" ht="165" x14ac:dyDescent="0.25">
@@ -5917,13 +5935,13 @@
         <v>122</v>
       </c>
       <c r="AB10" s="23" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="AC10" s="22" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="AD10" s="23" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="11" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -5979,7 +5997,7 @@
         <v>134</v>
       </c>
       <c r="V11" s="22" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="W11" s="16" t="s">
         <v>44</v>
@@ -6047,7 +6065,7 @@
         <v>134</v>
       </c>
       <c r="V12" s="22" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="W12" s="16" t="s">
         <v>44</v>
@@ -6115,13 +6133,13 @@
         <v>134</v>
       </c>
       <c r="V13" s="22" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="W13" s="16" t="s">
         <v>147</v>
       </c>
       <c r="X13" s="24" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="Y13" s="16" t="s">
         <v>147</v>
@@ -6183,7 +6201,7 @@
         <v>134</v>
       </c>
       <c r="V14" s="22" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="W14" s="16" t="s">
         <v>44</v>
@@ -6201,7 +6219,7 @@
         <v>155</v>
       </c>
       <c r="AC14" s="18" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -6257,7 +6275,7 @@
         <v>134</v>
       </c>
       <c r="V15" s="22" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="W15" s="16" t="s">
         <v>44</v>
@@ -6269,10 +6287,10 @@
         <v>92</v>
       </c>
       <c r="Z15" s="14" t="s">
+        <v>837</v>
+      </c>
+      <c r="AC15" s="22" t="s">
         <v>838</v>
-      </c>
-      <c r="AC15" s="22" t="s">
-        <v>839</v>
       </c>
     </row>
     <row r="16" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -6328,7 +6346,7 @@
         <v>134</v>
       </c>
       <c r="V16" s="22" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="W16" s="16" t="s">
         <v>44</v>
@@ -6340,10 +6358,10 @@
         <v>92</v>
       </c>
       <c r="Z16" s="14" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="AC16" s="22" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="17" spans="1:30" ht="255" x14ac:dyDescent="0.25">
@@ -6399,7 +6417,7 @@
         <v>134</v>
       </c>
       <c r="V17" s="22" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="W17" s="16" t="s">
         <v>147</v>
@@ -6467,7 +6485,7 @@
         <v>134</v>
       </c>
       <c r="V18" s="22" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="W18" s="16" t="s">
         <v>147</v>
@@ -6535,7 +6553,7 @@
         <v>134</v>
       </c>
       <c r="V19" s="22" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="W19" s="16" t="s">
         <v>44</v>
@@ -6600,7 +6618,7 @@
         <v>194</v>
       </c>
       <c r="V20" s="22" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="W20" s="25" t="s">
         <v>44</v>
@@ -6617,7 +6635,7 @@
       <c r="AA20" s="26"/>
       <c r="AB20" s="26"/>
       <c r="AC20" s="22" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="21" spans="1:30" ht="195" x14ac:dyDescent="0.25">
@@ -6670,7 +6688,7 @@
         <v>194</v>
       </c>
       <c r="V21" s="22" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="W21" s="16" t="s">
         <v>44</v>
@@ -6708,13 +6726,13 @@
         <v>206</v>
       </c>
       <c r="M22" s="18" t="s">
+        <v>849</v>
+      </c>
+      <c r="N22" s="18" t="s">
         <v>850</v>
       </c>
-      <c r="N22" s="18" t="s">
+      <c r="T22" s="22" t="s">
         <v>851</v>
-      </c>
-      <c r="T22" s="22" t="s">
-        <v>852</v>
       </c>
       <c r="W22" s="24" t="s">
         <v>44</v>
@@ -6726,13 +6744,13 @@
         <v>81</v>
       </c>
       <c r="Z22" s="22" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AB22" s="22" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="AD22" s="22" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="23" spans="1:30" ht="255" x14ac:dyDescent="0.25">
@@ -6891,7 +6909,7 @@
         <v>232</v>
       </c>
       <c r="V25" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="W25" s="16" t="s">
         <v>44</v>
@@ -6906,10 +6924,10 @@
         <v>233</v>
       </c>
       <c r="AA25" s="18" t="s">
+        <v>853</v>
+      </c>
+      <c r="AC25" s="22" t="s">
         <v>854</v>
-      </c>
-      <c r="AC25" s="22" t="s">
-        <v>855</v>
       </c>
     </row>
     <row r="26" spans="1:30" ht="180" x14ac:dyDescent="0.25">
@@ -6965,7 +6983,7 @@
         <v>246</v>
       </c>
       <c r="V26" s="22" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="W26" s="16" t="s">
         <v>44</v>
@@ -6980,7 +6998,7 @@
         <v>247</v>
       </c>
       <c r="AA26" s="18" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="27" spans="1:30" ht="135" x14ac:dyDescent="0.25">
@@ -7039,7 +7057,7 @@
         <v>262</v>
       </c>
       <c r="V27" s="22" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="W27" s="16" t="s">
         <v>44</v>
@@ -7169,7 +7187,7 @@
         <v>278</v>
       </c>
       <c r="V29" s="22" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="W29" s="16" t="s">
         <v>44</v>
@@ -7293,7 +7311,7 @@
         <v>292</v>
       </c>
       <c r="V31" s="22" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="W31" s="16" t="s">
         <v>44</v>
@@ -7358,7 +7376,7 @@
         <v>251</v>
       </c>
       <c r="V32" s="22" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="W32" s="16" t="s">
         <v>44</v>
@@ -7370,10 +7388,10 @@
         <v>81</v>
       </c>
       <c r="Z32" s="14" t="s">
-        <v>867</v>
+        <v>998</v>
       </c>
       <c r="AC32" s="22" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="33" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -7429,13 +7447,13 @@
         <v>81</v>
       </c>
       <c r="Z33" s="14" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="AC33" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
-    <row r="34" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="17">
         <v>33</v>
       </c>
@@ -7488,13 +7506,13 @@
         <v>81</v>
       </c>
       <c r="Z34" s="14" t="s">
-        <v>869</v>
+        <v>996</v>
       </c>
       <c r="AA34" s="18" t="s">
         <v>315</v>
       </c>
       <c r="AC34" s="22" t="s">
-        <v>859</v>
+        <v>997</v>
       </c>
     </row>
     <row r="35" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -7547,10 +7565,10 @@
         <v>81</v>
       </c>
       <c r="Z35" s="14" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
       <c r="AC35" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="36" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7609,7 +7627,7 @@
         <v>331</v>
       </c>
       <c r="V36" s="22" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="W36" s="16" t="s">
         <v>44</v>
@@ -7618,13 +7636,13 @@
         <v>80</v>
       </c>
       <c r="Y36" s="24" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="Z36" s="20" t="s">
         <v>332</v>
       </c>
       <c r="AC36" s="22" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="37" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7680,7 +7698,7 @@
         <v>331</v>
       </c>
       <c r="V37" s="22" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="W37" s="16" t="s">
         <v>44</v>
@@ -7689,13 +7707,13 @@
         <v>80</v>
       </c>
       <c r="Y37" s="24" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="Z37" s="20" t="s">
         <v>340</v>
       </c>
       <c r="AC37" s="22" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="38" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7751,7 +7769,7 @@
         <v>351</v>
       </c>
       <c r="V38" s="22" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="W38" s="16" t="s">
         <v>44</v>
@@ -7760,13 +7778,13 @@
         <v>80</v>
       </c>
       <c r="Y38" s="24" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="Z38" s="20" t="s">
         <v>352</v>
       </c>
       <c r="AC38" s="22" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="39" spans="1:30" x14ac:dyDescent="0.25">
@@ -7842,7 +7860,7 @@
         <v>51</v>
       </c>
       <c r="V40" s="22" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
       <c r="W40" s="16" t="s">
         <v>44</v>
@@ -7866,7 +7884,7 @@
         <v>365</v>
       </c>
       <c r="AD40" s="22" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="41" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -7922,13 +7940,13 @@
         <v>81</v>
       </c>
       <c r="Z41" s="14" t="s">
-        <v>873</v>
+        <v>870</v>
       </c>
       <c r="AA41" s="18" t="s">
         <v>375</v>
       </c>
       <c r="AC41" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="42" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -7984,10 +8002,10 @@
         <v>81</v>
       </c>
       <c r="Z42" s="14" t="s">
-        <v>874</v>
+        <v>871</v>
       </c>
       <c r="AC42" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="43" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8043,10 +8061,10 @@
         <v>81</v>
       </c>
       <c r="Z43" s="14" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
       <c r="AC43" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="44" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8102,10 +8120,10 @@
         <v>81</v>
       </c>
       <c r="Z44" s="14" t="s">
-        <v>876</v>
+        <v>873</v>
       </c>
       <c r="AC44" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="45" spans="1:30" x14ac:dyDescent="0.25">
@@ -8210,11 +8228,14 @@
       <c r="Y46" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="Z46" s="20" t="s">
+      <c r="Z46" s="14" t="s">
+        <v>992</v>
+      </c>
+      <c r="AA46" s="18" t="s">
         <v>409</v>
       </c>
-      <c r="AA46" s="18" t="s">
-        <v>410</v>
+      <c r="AC46" s="22" t="s">
+        <v>991</v>
       </c>
     </row>
     <row r="47" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8225,13 +8246,13 @@
         <v>33</v>
       </c>
       <c r="C47" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="D47" s="16" t="s">
         <v>411</v>
       </c>
-      <c r="D47" s="16" t="s">
-        <v>412</v>
-      </c>
       <c r="E47" s="16" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>205</v>
@@ -8240,16 +8261,16 @@
         <v>385</v>
       </c>
       <c r="M47" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="N47" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="O47" s="16" t="s">
         <v>413</v>
       </c>
-      <c r="N47" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="O47" s="16" t="s">
+      <c r="P47" s="16" t="s">
         <v>414</v>
-      </c>
-      <c r="P47" s="16" t="s">
-        <v>415</v>
       </c>
       <c r="S47" s="16" t="s">
         <v>104</v>
@@ -8270,10 +8291,10 @@
         <v>81</v>
       </c>
       <c r="Z47" s="14" t="s">
-        <v>877</v>
+        <v>874</v>
       </c>
       <c r="AC47" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8284,31 +8305,31 @@
         <v>33</v>
       </c>
       <c r="C48" s="7" t="s">
+        <v>415</v>
+      </c>
+      <c r="D48" s="16" t="s">
         <v>416</v>
       </c>
-      <c r="D48" s="16" t="s">
-        <v>417</v>
-      </c>
       <c r="E48" s="16" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>205</v>
       </c>
       <c r="G48" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="M48" s="18" t="s">
         <v>418</v>
       </c>
-      <c r="M48" s="18" t="s">
+      <c r="N48" s="18" t="s">
         <v>419</v>
       </c>
-      <c r="N48" s="18" t="s">
+      <c r="O48" s="16" t="s">
         <v>420</v>
       </c>
-      <c r="O48" s="16" t="s">
+      <c r="P48" s="16" t="s">
         <v>421</v>
-      </c>
-      <c r="P48" s="16" t="s">
-        <v>422</v>
       </c>
       <c r="S48" s="16" t="s">
         <v>104</v>
@@ -8317,7 +8338,7 @@
         <v>373</v>
       </c>
       <c r="U48" s="16" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="W48" s="16" t="s">
         <v>44</v>
@@ -8329,10 +8350,10 @@
         <v>81</v>
       </c>
       <c r="Z48" s="14" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
       <c r="AC48" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="49" spans="1:31" ht="30" x14ac:dyDescent="0.25">
@@ -8343,25 +8364,25 @@
         <v>33</v>
       </c>
       <c r="C49" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="D49" s="16" t="s">
         <v>424</v>
       </c>
-      <c r="D49" s="16" t="s">
-        <v>425</v>
-      </c>
       <c r="E49" s="16" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>205</v>
       </c>
       <c r="G49" s="7" t="s">
+        <v>425</v>
+      </c>
+      <c r="J49" s="7" t="s">
         <v>426</v>
       </c>
-      <c r="J49" s="7" t="s">
+      <c r="K49" s="7" t="s">
         <v>427</v>
-      </c>
-      <c r="K49" s="7" t="s">
-        <v>428</v>
       </c>
       <c r="M49" s="18" t="s">
         <v>51</v>
@@ -8379,10 +8400,10 @@
         <v>147</v>
       </c>
       <c r="AA49" s="18" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="AC49" s="18" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
     </row>
     <row r="50" spans="1:31" ht="45" x14ac:dyDescent="0.25">
@@ -8393,22 +8414,22 @@
         <v>33</v>
       </c>
       <c r="C50" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="D50" s="16" t="s">
         <v>430</v>
       </c>
-      <c r="D50" s="16" t="s">
-        <v>431</v>
-      </c>
       <c r="E50" s="16" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K50" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="L50" s="12" t="s">
         <v>432</v>
-      </c>
-      <c r="L50" s="12" t="s">
-        <v>433</v>
       </c>
       <c r="M50" s="18" t="s">
         <v>51</v>
@@ -8426,10 +8447,10 @@
         <v>147</v>
       </c>
       <c r="AA50" s="18" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="AC50" s="18" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="30" x14ac:dyDescent="0.25">
@@ -8440,25 +8461,25 @@
         <v>33</v>
       </c>
       <c r="C51" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="D51" s="16" t="s">
         <v>434</v>
       </c>
-      <c r="D51" s="16" t="s">
-        <v>435</v>
-      </c>
       <c r="E51" s="16" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>205</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="J51" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="K51" s="7" t="s">
         <v>436</v>
-      </c>
-      <c r="K51" s="7" t="s">
-        <v>437</v>
       </c>
       <c r="M51" s="18" t="s">
         <v>51</v>
@@ -8476,10 +8497,10 @@
         <v>147</v>
       </c>
       <c r="AA51" s="18" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="AC51" s="18" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="45" x14ac:dyDescent="0.25">
@@ -8490,25 +8511,25 @@
         <v>33</v>
       </c>
       <c r="C52" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="D52" s="16" t="s">
         <v>438</v>
       </c>
-      <c r="D52" s="16" t="s">
-        <v>439</v>
-      </c>
       <c r="E52" s="16" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F52" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J52" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="K52" s="7" t="s">
         <v>440</v>
       </c>
-      <c r="K52" s="7" t="s">
-        <v>441</v>
-      </c>
       <c r="L52" s="12" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="M52" s="18" t="s">
         <v>51</v>
@@ -8526,10 +8547,10 @@
         <v>147</v>
       </c>
       <c r="AA52" s="18" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="AC52" s="18" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
     </row>
     <row r="53" spans="1:31" ht="75" x14ac:dyDescent="0.25">
@@ -8540,28 +8561,28 @@
         <v>33</v>
       </c>
       <c r="C53" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="D53" s="16" t="s">
         <v>442</v>
       </c>
-      <c r="D53" s="16" t="s">
-        <v>443</v>
-      </c>
       <c r="E53" s="16" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>205</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="M53" s="18" t="s">
+        <v>814</v>
+      </c>
+      <c r="N53" s="18" t="s">
         <v>815</v>
       </c>
-      <c r="N53" s="18" t="s">
-        <v>816</v>
-      </c>
       <c r="V53" s="22" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="W53" s="24" t="s">
         <v>44</v>
@@ -8573,10 +8594,10 @@
         <v>302</v>
       </c>
       <c r="Z53" s="14" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="AC53" s="22" t="s">
-        <v>881</v>
+        <v>878</v>
       </c>
     </row>
     <row r="54" spans="1:31" ht="180" x14ac:dyDescent="0.25">
@@ -8587,46 +8608,46 @@
         <v>33</v>
       </c>
       <c r="C54" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="D54" s="16" t="s">
         <v>445</v>
       </c>
-      <c r="D54" s="16" t="s">
-        <v>446</v>
-      </c>
       <c r="E54" s="16" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>205</v>
       </c>
       <c r="G54" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="J54" s="7" t="s">
         <v>447</v>
       </c>
-      <c r="J54" s="7" t="s">
+      <c r="K54" s="7" t="s">
         <v>448</v>
       </c>
-      <c r="K54" s="7" t="s">
+      <c r="M54" s="18" t="s">
         <v>449</v>
       </c>
-      <c r="M54" s="18" t="s">
+      <c r="N54" s="18" t="s">
         <v>450</v>
       </c>
-      <c r="N54" s="18" t="s">
+      <c r="O54" s="16" t="s">
         <v>451</v>
       </c>
-      <c r="O54" s="16" t="s">
+      <c r="P54" s="16" t="s">
         <v>452</v>
-      </c>
-      <c r="P54" s="16" t="s">
-        <v>453</v>
       </c>
       <c r="S54" s="16" t="s">
         <v>104</v>
       </c>
       <c r="T54" s="18" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="V54" s="22" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="W54" s="16" t="s">
         <v>44</v>
@@ -8638,22 +8659,22 @@
         <v>81</v>
       </c>
       <c r="Z54" s="20" t="s">
+        <v>454</v>
+      </c>
+      <c r="AA54" s="18" t="s">
         <v>455</v>
       </c>
-      <c r="AA54" s="18" t="s">
+      <c r="AB54" s="18" t="s">
         <v>456</v>
       </c>
-      <c r="AB54" s="18" t="s">
+      <c r="AC54" s="22" t="s">
+        <v>879</v>
+      </c>
+      <c r="AD54" s="18" t="s">
         <v>457</v>
       </c>
-      <c r="AC54" s="22" t="s">
-        <v>882</v>
-      </c>
-      <c r="AD54" s="18" t="s">
+      <c r="AE54" s="16" t="s">
         <v>458</v>
-      </c>
-      <c r="AE54" s="16" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="55" spans="1:31" ht="90" x14ac:dyDescent="0.25">
@@ -8664,34 +8685,34 @@
         <v>33</v>
       </c>
       <c r="C55" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="D55" s="16" t="s">
         <v>460</v>
       </c>
-      <c r="D55" s="16" t="s">
-        <v>461</v>
-      </c>
       <c r="E55" s="16" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>63</v>
       </c>
       <c r="L55" s="12" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="M55" s="22" t="s">
+        <v>816</v>
+      </c>
+      <c r="N55" s="22" t="s">
         <v>817</v>
       </c>
-      <c r="N55" s="22" t="s">
+      <c r="P55" s="24" t="s">
+        <v>881</v>
+      </c>
+      <c r="T55" s="22" t="s">
         <v>818</v>
       </c>
-      <c r="P55" s="24" t="s">
-        <v>884</v>
-      </c>
-      <c r="T55" s="22" t="s">
-        <v>819</v>
-      </c>
       <c r="V55" s="27" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="W55" s="24" t="s">
         <v>44</v>
@@ -8703,10 +8724,10 @@
         <v>92</v>
       </c>
       <c r="Z55" s="14" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="AC55" s="27" t="s">
-        <v>971</v>
+        <v>965</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="120" x14ac:dyDescent="0.25">
@@ -8717,46 +8738,46 @@
         <v>33</v>
       </c>
       <c r="C56" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="D56" s="16" t="s">
         <v>463</v>
       </c>
-      <c r="D56" s="16" t="s">
-        <v>464</v>
-      </c>
       <c r="E56" s="16" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J56" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="K56" s="7" t="s">
         <v>465</v>
       </c>
-      <c r="K56" s="7" t="s">
+      <c r="L56" s="12" t="s">
         <v>466</v>
       </c>
-      <c r="L56" s="12" t="s">
+      <c r="M56" s="18" t="s">
         <v>467</v>
       </c>
-      <c r="M56" s="18" t="s">
+      <c r="N56" s="18" t="s">
         <v>468</v>
       </c>
-      <c r="N56" s="18" t="s">
+      <c r="O56" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="O56" s="16" t="s">
+      <c r="P56" s="16" t="s">
         <v>470</v>
-      </c>
-      <c r="P56" s="16" t="s">
-        <v>471</v>
       </c>
       <c r="S56" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T56" s="18" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="V56" s="22" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="W56" s="16" t="s">
         <v>44</v>
@@ -8768,7 +8789,7 @@
         <v>92</v>
       </c>
       <c r="Z56" s="20" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="57" spans="1:31" ht="90" x14ac:dyDescent="0.25">
@@ -8779,43 +8800,43 @@
         <v>33</v>
       </c>
       <c r="C57" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="D57" s="16" t="s">
         <v>474</v>
       </c>
-      <c r="D57" s="16" t="s">
-        <v>475</v>
-      </c>
       <c r="E57" s="16" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K57" s="7" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L57" s="12" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="M57" s="18" t="s">
+        <v>467</v>
+      </c>
+      <c r="N57" s="18" t="s">
         <v>468</v>
       </c>
-      <c r="N57" s="18" t="s">
+      <c r="O57" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="O57" s="16" t="s">
+      <c r="P57" s="16" t="s">
         <v>470</v>
-      </c>
-      <c r="P57" s="16" t="s">
-        <v>471</v>
       </c>
       <c r="S57" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T57" s="18" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="V57" s="22" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="W57" s="16" t="s">
         <v>44</v>
@@ -8827,7 +8848,7 @@
         <v>92</v>
       </c>
       <c r="Z57" s="14" t="s">
-        <v>972</v>
+        <v>966</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="75" x14ac:dyDescent="0.25">
@@ -8838,46 +8859,46 @@
         <v>33</v>
       </c>
       <c r="C58" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="D58" s="16" t="s">
         <v>477</v>
       </c>
-      <c r="D58" s="16" t="s">
-        <v>478</v>
-      </c>
       <c r="E58" s="16" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>205</v>
       </c>
       <c r="G58" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="J58" s="7" t="s">
         <v>479</v>
       </c>
-      <c r="J58" s="7" t="s">
+      <c r="K58" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="M58" s="18" t="s">
         <v>480</v>
       </c>
-      <c r="K58" s="7" t="s">
-        <v>466</v>
-      </c>
-      <c r="M58" s="18" t="s">
+      <c r="N58" s="18" t="s">
         <v>481</v>
       </c>
-      <c r="N58" s="18" t="s">
+      <c r="O58" s="16" t="s">
+        <v>469</v>
+      </c>
+      <c r="P58" s="16" t="s">
         <v>482</v>
-      </c>
-      <c r="O58" s="16" t="s">
-        <v>470</v>
-      </c>
-      <c r="P58" s="16" t="s">
-        <v>483</v>
       </c>
       <c r="S58" s="16" t="s">
         <v>104</v>
       </c>
       <c r="T58" s="18" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="V58" s="22" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="W58" s="16" t="s">
         <v>44</v>
@@ -8889,13 +8910,13 @@
         <v>81</v>
       </c>
       <c r="Z58" s="22" t="s">
-        <v>973</v>
+        <v>967</v>
       </c>
       <c r="AA58" s="18" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="AC58" s="18" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
     </row>
     <row r="59" spans="1:31" ht="45" x14ac:dyDescent="0.25">
@@ -8906,13 +8927,13 @@
         <v>33</v>
       </c>
       <c r="C59" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="D59" s="16" t="s">
         <v>485</v>
       </c>
-      <c r="D59" s="16" t="s">
-        <v>486</v>
-      </c>
       <c r="E59" s="16" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>205</v>
@@ -8921,22 +8942,22 @@
         <v>206</v>
       </c>
       <c r="M59" s="18" t="s">
+        <v>486</v>
+      </c>
+      <c r="N59" s="18" t="s">
         <v>487</v>
       </c>
-      <c r="N59" s="18" t="s">
+      <c r="O59" s="16" t="s">
         <v>488</v>
       </c>
-      <c r="O59" s="16" t="s">
+      <c r="P59" s="16" t="s">
         <v>489</v>
-      </c>
-      <c r="P59" s="16" t="s">
-        <v>490</v>
       </c>
       <c r="S59" s="16" t="s">
         <v>104</v>
       </c>
       <c r="T59" s="18" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="W59" s="16" t="s">
         <v>44</v>
@@ -8948,7 +8969,7 @@
         <v>81</v>
       </c>
       <c r="Z59" s="20" t="s">
-        <v>974</v>
+        <v>968</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="195" x14ac:dyDescent="0.25">
@@ -8959,40 +8980,40 @@
         <v>33</v>
       </c>
       <c r="C60" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="D60" s="16" t="s">
         <v>492</v>
       </c>
-      <c r="D60" s="16" t="s">
-        <v>493</v>
-      </c>
       <c r="E60" s="16" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J60" s="12" t="s">
+        <v>493</v>
+      </c>
+      <c r="L60" s="12" t="s">
         <v>494</v>
       </c>
-      <c r="L60" s="12" t="s">
-        <v>495</v>
-      </c>
       <c r="M60" s="18" t="s">
+        <v>486</v>
+      </c>
+      <c r="N60" s="18" t="s">
         <v>487</v>
       </c>
-      <c r="N60" s="18" t="s">
+      <c r="O60" s="16" t="s">
         <v>488</v>
       </c>
-      <c r="O60" s="16" t="s">
+      <c r="P60" s="16" t="s">
         <v>489</v>
-      </c>
-      <c r="P60" s="16" t="s">
-        <v>490</v>
       </c>
       <c r="S60" s="16" t="s">
         <v>104</v>
       </c>
       <c r="T60" s="18" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="W60" s="16" t="s">
         <v>44</v>
@@ -9004,7 +9025,7 @@
         <v>81</v>
       </c>
       <c r="Z60" s="20" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="61" spans="1:31" ht="195" x14ac:dyDescent="0.25">
@@ -9015,35 +9036,35 @@
         <v>33</v>
       </c>
       <c r="C61" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="D61" s="16" t="s">
         <v>497</v>
       </c>
-      <c r="D61" s="16" t="s">
+      <c r="E61" s="16" t="s">
         <v>498</v>
-      </c>
-      <c r="E61" s="16" t="s">
-        <v>499</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K61" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="L61" s="12" t="s">
         <v>500</v>
-      </c>
-      <c r="L61" s="12" t="s">
-        <v>501</v>
       </c>
       <c r="M61" s="18" t="s">
         <v>51</v>
       </c>
       <c r="T61" s="21"/>
       <c r="V61" s="22" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="W61" s="16" t="s">
         <v>147</v>
       </c>
       <c r="X61" s="16" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="Y61" s="16" t="s">
         <v>147</v>
@@ -9052,16 +9073,16 @@
         <v>147</v>
       </c>
       <c r="AA61" s="18" t="s">
+        <v>503</v>
+      </c>
+      <c r="AB61" s="22" t="s">
         <v>504</v>
       </c>
-      <c r="AB61" s="22" t="s">
-        <v>505</v>
-      </c>
       <c r="AC61" s="22" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="AD61" s="23" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="62" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
@@ -9072,43 +9093,43 @@
         <v>33</v>
       </c>
       <c r="C62" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="D62" s="16" t="s">
         <v>506</v>
       </c>
-      <c r="D62" s="16" t="s">
-        <v>507</v>
-      </c>
       <c r="E62" s="16" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J62" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="L62" s="12" t="s">
         <v>508</v>
       </c>
-      <c r="L62" s="12" t="s">
+      <c r="M62" s="18" t="s">
         <v>509</v>
       </c>
-      <c r="M62" s="18" t="s">
+      <c r="N62" s="18" t="s">
         <v>510</v>
       </c>
-      <c r="N62" s="18" t="s">
+      <c r="O62" s="16" t="s">
         <v>511</v>
       </c>
-      <c r="O62" s="16" t="s">
+      <c r="P62" s="16" t="s">
         <v>512</v>
       </c>
-      <c r="P62" s="16" t="s">
+      <c r="S62" s="16" t="s">
+        <v>501</v>
+      </c>
+      <c r="T62" s="18" t="s">
         <v>513</v>
       </c>
-      <c r="S62" s="16" t="s">
-        <v>502</v>
-      </c>
-      <c r="T62" s="18" t="s">
-        <v>514</v>
-      </c>
       <c r="V62" s="22" t="s">
-        <v>892</v>
+        <v>993</v>
       </c>
       <c r="W62" s="16" t="s">
         <v>44</v>
@@ -9120,10 +9141,10 @@
         <v>81</v>
       </c>
       <c r="Z62" s="20" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AC62" s="22" t="s">
-        <v>911</v>
+        <v>905</v>
       </c>
     </row>
     <row r="63" spans="1:31" ht="135" x14ac:dyDescent="0.25">
@@ -9134,40 +9155,40 @@
         <v>33</v>
       </c>
       <c r="C63" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="D63" s="16" t="s">
         <v>516</v>
       </c>
-      <c r="D63" s="16" t="s">
-        <v>517</v>
-      </c>
       <c r="E63" s="16" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>63</v>
       </c>
       <c r="L63" s="12" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="M63" s="18" t="s">
+        <v>517</v>
+      </c>
+      <c r="N63" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="N63" s="18" t="s">
+      <c r="O63" s="16" t="s">
+        <v>511</v>
+      </c>
+      <c r="P63" s="16" t="s">
         <v>519</v>
-      </c>
-      <c r="O63" s="16" t="s">
-        <v>512</v>
-      </c>
-      <c r="P63" s="16" t="s">
-        <v>520</v>
       </c>
       <c r="S63" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T63" s="18" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="V63" s="22" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="W63" s="16" t="s">
         <v>44</v>
@@ -9179,7 +9200,7 @@
         <v>92</v>
       </c>
       <c r="Z63" s="20" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="64" spans="1:31" ht="135" x14ac:dyDescent="0.25">
@@ -9190,40 +9211,40 @@
         <v>33</v>
       </c>
       <c r="C64" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="D64" s="16" t="s">
         <v>523</v>
       </c>
-      <c r="D64" s="16" t="s">
-        <v>524</v>
-      </c>
       <c r="E64" s="16" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="F64" s="7" t="s">
         <v>63</v>
       </c>
       <c r="L64" s="12" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="M64" s="18" t="s">
+        <v>524</v>
+      </c>
+      <c r="N64" s="18" t="s">
         <v>525</v>
       </c>
-      <c r="N64" s="18" t="s">
+      <c r="O64" s="16" t="s">
+        <v>511</v>
+      </c>
+      <c r="P64" s="16" t="s">
         <v>526</v>
-      </c>
-      <c r="O64" s="16" t="s">
-        <v>512</v>
-      </c>
-      <c r="P64" s="16" t="s">
-        <v>527</v>
       </c>
       <c r="S64" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T64" s="18" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="V64" s="22" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="W64" s="16" t="s">
         <v>44</v>
@@ -9235,7 +9256,7 @@
         <v>92</v>
       </c>
       <c r="Z64" s="20" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="65" spans="1:30" ht="165" x14ac:dyDescent="0.25">
@@ -9246,19 +9267,19 @@
         <v>33</v>
       </c>
       <c r="C65" s="7" t="s">
+        <v>527</v>
+      </c>
+      <c r="D65" s="16" t="s">
         <v>528</v>
       </c>
-      <c r="D65" s="16" t="s">
+      <c r="E65" s="16" t="s">
         <v>529</v>
-      </c>
-      <c r="E65" s="16" t="s">
-        <v>530</v>
       </c>
       <c r="F65" s="7" t="s">
         <v>63</v>
       </c>
       <c r="L65" s="12" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="M65" s="18" t="s">
         <v>51</v>
@@ -9284,43 +9305,43 @@
         <v>33</v>
       </c>
       <c r="C66" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="D66" s="16" t="s">
         <v>532</v>
       </c>
-      <c r="D66" s="16" t="s">
+      <c r="E66" s="16" t="s">
         <v>533</v>
-      </c>
-      <c r="E66" s="16" t="s">
-        <v>534</v>
       </c>
       <c r="F66" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J66" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="L66" s="12" t="s">
         <v>508</v>
       </c>
-      <c r="L66" s="12" t="s">
-        <v>509</v>
-      </c>
       <c r="M66" s="18" t="s">
+        <v>534</v>
+      </c>
+      <c r="N66" s="18" t="s">
         <v>535</v>
       </c>
-      <c r="N66" s="18" t="s">
+      <c r="O66" s="16" t="s">
         <v>536</v>
       </c>
-      <c r="O66" s="16" t="s">
+      <c r="P66" s="16" t="s">
         <v>537</v>
-      </c>
-      <c r="P66" s="16" t="s">
-        <v>538</v>
       </c>
       <c r="S66" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T66" s="18" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="V66" s="22" t="s">
-        <v>893</v>
+        <v>994</v>
       </c>
       <c r="W66" s="16" t="s">
         <v>44</v>
@@ -9332,10 +9353,10 @@
         <v>81</v>
       </c>
       <c r="Z66" s="20" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="AC66" s="22" t="s">
-        <v>911</v>
+        <v>905</v>
       </c>
     </row>
     <row r="67" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -9346,43 +9367,43 @@
         <v>33</v>
       </c>
       <c r="C67" s="7" t="s">
+        <v>539</v>
+      </c>
+      <c r="D67" s="16" t="s">
         <v>540</v>
       </c>
-      <c r="D67" s="16" t="s">
+      <c r="E67" s="16" t="s">
         <v>541</v>
-      </c>
-      <c r="E67" s="16" t="s">
-        <v>542</v>
       </c>
       <c r="F67" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J67" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="L67" s="12" t="s">
         <v>508</v>
       </c>
-      <c r="L67" s="12" t="s">
-        <v>509</v>
-      </c>
       <c r="M67" s="18" t="s">
+        <v>542</v>
+      </c>
+      <c r="N67" s="18" t="s">
         <v>543</v>
       </c>
-      <c r="N67" s="18" t="s">
+      <c r="O67" s="16" t="s">
         <v>544</v>
       </c>
-      <c r="O67" s="16" t="s">
+      <c r="P67" s="16" t="s">
         <v>545</v>
-      </c>
-      <c r="P67" s="16" t="s">
-        <v>546</v>
       </c>
       <c r="S67" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T67" s="21" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="V67" s="22" t="s">
-        <v>894</v>
+        <v>995</v>
       </c>
       <c r="W67" s="16" t="s">
         <v>44</v>
@@ -9394,10 +9415,10 @@
         <v>81</v>
       </c>
       <c r="Z67" s="20" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AC67" s="22" t="s">
-        <v>911</v>
+        <v>905</v>
       </c>
     </row>
     <row r="68" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -9408,13 +9429,13 @@
         <v>33</v>
       </c>
       <c r="C68" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="D68" s="16" t="s">
         <v>548</v>
       </c>
-      <c r="D68" s="16" t="s">
-        <v>549</v>
-      </c>
       <c r="E68" s="16" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F68" s="7" t="s">
         <v>205</v>
@@ -9423,7 +9444,7 @@
         <v>206</v>
       </c>
       <c r="J68" s="7" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="M68" s="18" t="s">
         <v>51</v>
@@ -9441,10 +9462,10 @@
         <v>147</v>
       </c>
       <c r="AB68" s="22" t="s">
-        <v>895</v>
+        <v>889</v>
       </c>
       <c r="AD68" s="23" t="s">
-        <v>896</v>
+        <v>890</v>
       </c>
     </row>
     <row r="69" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -9455,19 +9476,19 @@
         <v>33</v>
       </c>
       <c r="C69" s="7" t="s">
+        <v>549</v>
+      </c>
+      <c r="D69" s="16" t="s">
         <v>550</v>
       </c>
-      <c r="D69" s="16" t="s">
+      <c r="E69" s="16" t="s">
         <v>551</v>
-      </c>
-      <c r="E69" s="16" t="s">
-        <v>552</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>63</v>
       </c>
       <c r="L69" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="M69" s="18" t="s">
         <v>51</v>
@@ -9485,10 +9506,10 @@
         <v>147</v>
       </c>
       <c r="AB69" s="22" t="s">
-        <v>895</v>
+        <v>889</v>
       </c>
       <c r="AD69" s="23" t="s">
-        <v>896</v>
+        <v>890</v>
       </c>
     </row>
     <row r="70" spans="1:30" ht="180" x14ac:dyDescent="0.25">
@@ -9499,43 +9520,43 @@
         <v>33</v>
       </c>
       <c r="C70" s="7" t="s">
+        <v>553</v>
+      </c>
+      <c r="D70" s="16" t="s">
         <v>554</v>
       </c>
-      <c r="D70" s="16" t="s">
+      <c r="E70" s="16" t="s">
         <v>555</v>
-      </c>
-      <c r="E70" s="16" t="s">
-        <v>556</v>
       </c>
       <c r="F70" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K70" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="L70" s="12" t="s">
         <v>557</v>
       </c>
-      <c r="L70" s="12" t="s">
+      <c r="M70" s="18" t="s">
         <v>558</v>
       </c>
-      <c r="M70" s="18" t="s">
+      <c r="N70" s="18" t="s">
         <v>559</v>
       </c>
-      <c r="N70" s="18" t="s">
+      <c r="O70" s="16" t="s">
         <v>560</v>
       </c>
-      <c r="O70" s="16" t="s">
+      <c r="P70" s="16" t="s">
         <v>561</v>
-      </c>
-      <c r="P70" s="16" t="s">
-        <v>562</v>
       </c>
       <c r="S70" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T70" s="18" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="V70" s="22" t="s">
-        <v>975</v>
+        <v>969</v>
       </c>
       <c r="W70" s="16" t="s">
         <v>44</v>
@@ -9547,10 +9568,10 @@
         <v>92</v>
       </c>
       <c r="Z70" s="20" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AC70" s="22" t="s">
-        <v>911</v>
+        <v>905</v>
       </c>
     </row>
     <row r="71" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -9561,40 +9582,40 @@
         <v>33</v>
       </c>
       <c r="C71" s="7" t="s">
+        <v>564</v>
+      </c>
+      <c r="D71" s="16" t="s">
         <v>565</v>
       </c>
-      <c r="D71" s="16" t="s">
+      <c r="E71" s="16" t="s">
         <v>566</v>
-      </c>
-      <c r="E71" s="16" t="s">
-        <v>567</v>
       </c>
       <c r="F71" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="L71" s="12" t="s">
+        <v>567</v>
+      </c>
+      <c r="M71" s="18" t="s">
         <v>568</v>
       </c>
-      <c r="M71" s="18" t="s">
+      <c r="N71" s="18" t="s">
         <v>569</v>
       </c>
-      <c r="N71" s="18" t="s">
+      <c r="O71" s="16" t="s">
         <v>570</v>
       </c>
-      <c r="O71" s="16" t="s">
+      <c r="P71" s="16" t="s">
         <v>571</v>
-      </c>
-      <c r="P71" s="16" t="s">
-        <v>572</v>
       </c>
       <c r="S71" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T71" s="21" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="W71" s="16" t="s">
         <v>44</v>
@@ -9606,10 +9627,10 @@
         <v>92</v>
       </c>
       <c r="Z71" s="20" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="AC71" s="22" t="s">
-        <v>911</v>
+        <v>905</v>
       </c>
     </row>
     <row r="72" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -9620,46 +9641,46 @@
         <v>33</v>
       </c>
       <c r="C72" s="7" t="s">
+        <v>574</v>
+      </c>
+      <c r="D72" s="16" t="s">
         <v>575</v>
       </c>
-      <c r="D72" s="16" t="s">
+      <c r="E72" s="16" t="s">
         <v>576</v>
-      </c>
-      <c r="E72" s="16" t="s">
-        <v>577</v>
       </c>
       <c r="F72" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J72" s="7" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="L72" s="12" t="s">
         <v>121</v>
       </c>
       <c r="M72" s="18" t="s">
+        <v>578</v>
+      </c>
+      <c r="N72" s="18" t="s">
         <v>579</v>
       </c>
-      <c r="N72" s="18" t="s">
+      <c r="O72" s="16" t="s">
+        <v>560</v>
+      </c>
+      <c r="P72" s="16" t="s">
         <v>580</v>
-      </c>
-      <c r="O72" s="16" t="s">
-        <v>561</v>
-      </c>
-      <c r="P72" s="16" t="s">
-        <v>581</v>
       </c>
       <c r="S72" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T72" s="18" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="V72" s="22" t="s">
-        <v>897</v>
+        <v>891</v>
       </c>
       <c r="W72" s="16" t="s">
         <v>44</v>
@@ -9671,10 +9692,10 @@
         <v>81</v>
       </c>
       <c r="Z72" s="20" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AC72" s="22" t="s">
-        <v>911</v>
+        <v>905</v>
       </c>
     </row>
     <row r="73" spans="1:30" ht="135" x14ac:dyDescent="0.25">
@@ -9685,43 +9706,43 @@
         <v>33</v>
       </c>
       <c r="C73" s="7" t="s">
+        <v>582</v>
+      </c>
+      <c r="D73" s="16" t="s">
         <v>583</v>
       </c>
-      <c r="D73" s="16" t="s">
+      <c r="E73" s="16" t="s">
         <v>584</v>
-      </c>
-      <c r="E73" s="16" t="s">
-        <v>585</v>
       </c>
       <c r="F73" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J73" s="7" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="L73" s="12" t="s">
         <v>121</v>
       </c>
       <c r="M73" s="18" t="s">
+        <v>586</v>
+      </c>
+      <c r="N73" s="18" t="s">
         <v>587</v>
       </c>
-      <c r="N73" s="18" t="s">
+      <c r="O73" s="16" t="s">
         <v>588</v>
       </c>
-      <c r="O73" s="16" t="s">
+      <c r="P73" s="16" t="s">
         <v>589</v>
-      </c>
-      <c r="P73" s="16" t="s">
-        <v>590</v>
       </c>
       <c r="S73" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T73" s="18" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="V73" s="27" t="s">
-        <v>912</v>
+        <v>906</v>
       </c>
       <c r="W73" s="16" t="s">
         <v>44</v>
@@ -9733,10 +9754,10 @@
         <v>81</v>
       </c>
       <c r="Z73" s="20" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="AC73" s="27" t="s">
-        <v>913</v>
+        <v>907</v>
       </c>
     </row>
     <row r="74" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -9747,46 +9768,46 @@
         <v>33</v>
       </c>
       <c r="C74" s="7" t="s">
+        <v>592</v>
+      </c>
+      <c r="D74" s="16" t="s">
         <v>593</v>
       </c>
-      <c r="D74" s="16" t="s">
+      <c r="E74" s="16" t="s">
         <v>594</v>
-      </c>
-      <c r="E74" s="16" t="s">
-        <v>595</v>
       </c>
       <c r="F74" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J74" s="7" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="L74" s="12" t="s">
         <v>121</v>
       </c>
       <c r="M74" s="18" t="s">
+        <v>596</v>
+      </c>
+      <c r="N74" s="18" t="s">
         <v>597</v>
       </c>
-      <c r="N74" s="18" t="s">
-        <v>598</v>
-      </c>
       <c r="O74" s="16" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="P74" s="16" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="S74" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T74" s="18" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="V74" s="22" t="s">
-        <v>897</v>
+        <v>891</v>
       </c>
       <c r="W74" s="16" t="s">
         <v>44</v>
@@ -9798,10 +9819,10 @@
         <v>81</v>
       </c>
       <c r="Z74" s="20" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="AC74" s="22" t="s">
-        <v>911</v>
+        <v>905</v>
       </c>
     </row>
     <row r="75" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -9812,31 +9833,31 @@
         <v>33</v>
       </c>
       <c r="C75" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="D75" s="16" t="s">
         <v>600</v>
       </c>
-      <c r="D75" s="16" t="s">
+      <c r="E75" s="16" t="s">
         <v>601</v>
-      </c>
-      <c r="E75" s="16" t="s">
-        <v>602</v>
       </c>
       <c r="F75" s="7" t="s">
         <v>205</v>
       </c>
       <c r="J75" s="7" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="M75" s="22" t="s">
-        <v>976</v>
+        <v>970</v>
       </c>
       <c r="N75" s="22" t="s">
-        <v>977</v>
+        <v>971</v>
       </c>
       <c r="O75" s="24" t="s">
+        <v>605</v>
+      </c>
+      <c r="P75" s="24" t="s">
         <v>606</v>
-      </c>
-      <c r="P75" s="24" t="s">
-        <v>607</v>
       </c>
       <c r="Q75" s="24"/>
       <c r="R75" s="24"/>
@@ -9844,7 +9865,7 @@
         <v>43</v>
       </c>
       <c r="T75" s="33" t="s">
-        <v>979</v>
+        <v>973</v>
       </c>
       <c r="W75" s="32" t="s">
         <v>44</v>
@@ -9856,13 +9877,13 @@
         <v>81</v>
       </c>
       <c r="Z75" s="14" t="s">
-        <v>980</v>
+        <v>974</v>
       </c>
       <c r="AA75" s="22" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="AC75" s="22" t="s">
-        <v>978</v>
+        <v>972</v>
       </c>
     </row>
     <row r="76" spans="1:30" ht="225" x14ac:dyDescent="0.25">
@@ -9873,37 +9894,37 @@
         <v>33</v>
       </c>
       <c r="C76" s="7" t="s">
+        <v>609</v>
+      </c>
+      <c r="D76" s="16" t="s">
         <v>610</v>
       </c>
-      <c r="D76" s="16" t="s">
+      <c r="E76" s="16" t="s">
         <v>611</v>
-      </c>
-      <c r="E76" s="16" t="s">
-        <v>612</v>
       </c>
       <c r="F76" s="7" t="s">
         <v>63</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="M76" s="18" t="s">
+        <v>603</v>
+      </c>
+      <c r="N76" s="18" t="s">
         <v>604</v>
       </c>
-      <c r="N76" s="18" t="s">
+      <c r="O76" s="16" t="s">
         <v>605</v>
       </c>
-      <c r="O76" s="16" t="s">
+      <c r="P76" s="16" t="s">
         <v>606</v>
-      </c>
-      <c r="P76" s="16" t="s">
-        <v>607</v>
       </c>
       <c r="S76" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T76" s="18" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="W76" s="16" t="s">
         <v>44</v>
@@ -9912,13 +9933,13 @@
         <v>80</v>
       </c>
       <c r="Y76" s="24" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="Z76" s="20" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AC76" s="22" t="s">
-        <v>898</v>
+        <v>892</v>
       </c>
     </row>
     <row r="77" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -9929,40 +9950,40 @@
         <v>33</v>
       </c>
       <c r="C77" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="D77" s="16" t="s">
         <v>615</v>
       </c>
-      <c r="D77" s="16" t="s">
-        <v>616</v>
-      </c>
       <c r="E77" s="16" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="F77" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K77" s="7" t="s">
+        <v>616</v>
+      </c>
+      <c r="L77" s="12" t="s">
         <v>617</v>
       </c>
-      <c r="L77" s="12" t="s">
+      <c r="M77" s="18" t="s">
         <v>618</v>
       </c>
-      <c r="M77" s="18" t="s">
+      <c r="N77" s="18" t="s">
         <v>619</v>
       </c>
-      <c r="N77" s="18" t="s">
+      <c r="O77" s="16" t="s">
+        <v>605</v>
+      </c>
+      <c r="P77" s="16" t="s">
         <v>620</v>
-      </c>
-      <c r="O77" s="16" t="s">
-        <v>606</v>
-      </c>
-      <c r="P77" s="16" t="s">
-        <v>621</v>
       </c>
       <c r="S77" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T77" s="18" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="W77" s="16" t="s">
         <v>44</v>
@@ -9974,7 +9995,7 @@
         <v>92</v>
       </c>
       <c r="Z77" s="28" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="78" spans="1:30" ht="135" x14ac:dyDescent="0.25">
@@ -9985,37 +10006,37 @@
         <v>33</v>
       </c>
       <c r="C78" s="7" t="s">
+        <v>623</v>
+      </c>
+      <c r="D78" s="16" t="s">
         <v>624</v>
       </c>
-      <c r="D78" s="16" t="s">
+      <c r="E78" s="16" t="s">
         <v>625</v>
-      </c>
-      <c r="E78" s="16" t="s">
-        <v>626</v>
       </c>
       <c r="F78" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J78" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="K78" s="7" t="s">
         <v>627</v>
       </c>
-      <c r="K78" s="7" t="s">
+      <c r="L78" s="12" t="s">
         <v>628</v>
       </c>
-      <c r="L78" s="12" t="s">
+      <c r="M78" s="22" t="s">
+        <v>900</v>
+      </c>
+      <c r="N78" s="22" t="s">
+        <v>899</v>
+      </c>
+      <c r="O78" s="24" t="s">
         <v>629</v>
       </c>
-      <c r="M78" s="22" t="s">
-        <v>906</v>
-      </c>
-      <c r="N78" s="22" t="s">
-        <v>905</v>
-      </c>
-      <c r="O78" s="24" t="s">
+      <c r="P78" s="24" t="s">
         <v>630</v>
-      </c>
-      <c r="P78" s="24" t="s">
-        <v>631</v>
       </c>
       <c r="Q78" s="24"/>
       <c r="R78" s="24"/>
@@ -10023,10 +10044,10 @@
         <v>43</v>
       </c>
       <c r="T78" s="31" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="V78" s="22" t="s">
-        <v>901</v>
+        <v>895</v>
       </c>
       <c r="W78" s="16" t="s">
         <v>44</v>
@@ -10038,10 +10059,10 @@
         <v>81</v>
       </c>
       <c r="Z78" s="14" t="s">
-        <v>908</v>
+        <v>902</v>
       </c>
       <c r="AC78" s="22" t="s">
-        <v>907</v>
+        <v>901</v>
       </c>
     </row>
     <row r="79" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -10052,37 +10073,37 @@
         <v>33</v>
       </c>
       <c r="C79" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="D79" s="16" t="s">
         <v>633</v>
       </c>
-      <c r="D79" s="16" t="s">
+      <c r="E79" s="16" t="s">
         <v>634</v>
-      </c>
-      <c r="E79" s="16" t="s">
-        <v>635</v>
       </c>
       <c r="F79" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I79" s="7" t="s">
+        <v>635</v>
+      </c>
+      <c r="J79" s="7" t="s">
         <v>636</v>
       </c>
-      <c r="J79" s="7" t="s">
-        <v>637</v>
-      </c>
       <c r="L79" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M79" s="22" t="s">
-        <v>986</v>
+        <v>980</v>
       </c>
       <c r="N79" s="22" t="s">
-        <v>981</v>
+        <v>975</v>
       </c>
       <c r="T79" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V79" s="22" t="s">
-        <v>900</v>
+        <v>894</v>
       </c>
       <c r="W79" s="24" t="s">
         <v>44</v>
@@ -10094,13 +10115,13 @@
         <v>81</v>
       </c>
       <c r="Z79" s="14" t="s">
-        <v>990</v>
+        <v>984</v>
       </c>
       <c r="AB79" s="22" t="s">
-        <v>902</v>
+        <v>896</v>
       </c>
       <c r="AD79" s="23" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="80" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -10111,37 +10132,37 @@
         <v>33</v>
       </c>
       <c r="C80" s="7" t="s">
+        <v>637</v>
+      </c>
+      <c r="D80" s="16" t="s">
         <v>638</v>
       </c>
-      <c r="D80" s="16" t="s">
+      <c r="E80" s="16" t="s">
         <v>639</v>
-      </c>
-      <c r="E80" s="16" t="s">
-        <v>640</v>
       </c>
       <c r="F80" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I80" s="7" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="J80" s="7" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="L80" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M80" s="22" t="s">
-        <v>987</v>
+        <v>981</v>
       </c>
       <c r="N80" s="22" t="s">
-        <v>982</v>
+        <v>976</v>
       </c>
       <c r="T80" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V80" s="22" t="s">
-        <v>900</v>
+        <v>894</v>
       </c>
       <c r="W80" s="24" t="s">
         <v>44</v>
@@ -10153,16 +10174,16 @@
         <v>81</v>
       </c>
       <c r="Z80" s="14" t="s">
-        <v>991</v>
+        <v>985</v>
       </c>
       <c r="AB80" s="22" t="s">
-        <v>902</v>
+        <v>896</v>
       </c>
       <c r="AC80" s="22" t="s">
-        <v>984</v>
+        <v>978</v>
       </c>
       <c r="AD80" s="23" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="81" spans="1:33" ht="90" x14ac:dyDescent="0.25">
@@ -10173,37 +10194,37 @@
         <v>33</v>
       </c>
       <c r="C81" s="7" t="s">
+        <v>641</v>
+      </c>
+      <c r="D81" s="16" t="s">
         <v>642</v>
       </c>
-      <c r="D81" s="16" t="s">
+      <c r="E81" s="16" t="s">
         <v>643</v>
-      </c>
-      <c r="E81" s="16" t="s">
-        <v>644</v>
       </c>
       <c r="F81" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I81" s="7" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="J81" s="7" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="L81" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M81" s="22" t="s">
-        <v>988</v>
+        <v>982</v>
       </c>
       <c r="N81" s="22" t="s">
-        <v>985</v>
+        <v>979</v>
       </c>
       <c r="T81" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V81" s="22" t="s">
-        <v>920</v>
+        <v>914</v>
       </c>
       <c r="W81" s="24" t="s">
         <v>44</v>
@@ -10215,16 +10236,16 @@
         <v>81</v>
       </c>
       <c r="Z81" s="14" t="s">
-        <v>992</v>
+        <v>986</v>
       </c>
       <c r="AB81" s="22" t="s">
-        <v>902</v>
+        <v>896</v>
       </c>
       <c r="AC81" s="27" t="s">
-        <v>903</v>
+        <v>897</v>
       </c>
       <c r="AD81" s="23" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="82" spans="1:33" ht="45" x14ac:dyDescent="0.25">
@@ -10235,46 +10256,46 @@
         <v>33</v>
       </c>
       <c r="C82" s="7" t="s">
+        <v>645</v>
+      </c>
+      <c r="D82" s="16" t="s">
         <v>646</v>
       </c>
-      <c r="D82" s="16" t="s">
+      <c r="E82" s="16" t="s">
         <v>647</v>
-      </c>
-      <c r="E82" s="16" t="s">
-        <v>648</v>
       </c>
       <c r="F82" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I82" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="J82" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="L82" s="12" t="s">
+        <v>628</v>
+      </c>
+      <c r="M82" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="J82" s="7" t="s">
-        <v>637</v>
-      </c>
-      <c r="L82" s="12" t="s">
+      <c r="N82" s="18" t="s">
+        <v>650</v>
+      </c>
+      <c r="O82" s="16" t="s">
         <v>629</v>
       </c>
-      <c r="M82" s="18" t="s">
-        <v>650</v>
-      </c>
-      <c r="N82" s="18" t="s">
+      <c r="P82" s="16" t="s">
         <v>651</v>
-      </c>
-      <c r="O82" s="16" t="s">
-        <v>630</v>
-      </c>
-      <c r="P82" s="16" t="s">
-        <v>652</v>
       </c>
       <c r="S82" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T82" s="18" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="V82" s="22" t="s">
-        <v>901</v>
+        <v>895</v>
       </c>
       <c r="W82" s="16" t="s">
         <v>44</v>
@@ -10286,16 +10307,16 @@
         <v>92</v>
       </c>
       <c r="Z82" s="14" t="s">
-        <v>904</v>
+        <v>898</v>
       </c>
       <c r="AB82" s="22" t="s">
-        <v>902</v>
+        <v>896</v>
       </c>
       <c r="AC82" s="22" t="s">
-        <v>984</v>
+        <v>978</v>
       </c>
       <c r="AD82" s="23" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="83" spans="1:33" ht="75" x14ac:dyDescent="0.25">
@@ -10306,37 +10327,37 @@
         <v>33</v>
       </c>
       <c r="C83" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="D83" s="16" t="s">
         <v>655</v>
       </c>
-      <c r="D83" s="16" t="s">
+      <c r="E83" s="16" t="s">
         <v>656</v>
-      </c>
-      <c r="E83" s="16" t="s">
-        <v>657</v>
       </c>
       <c r="F83" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I83" s="7" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="J83" s="7" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="L83" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M83" s="22" t="s">
-        <v>989</v>
+        <v>983</v>
       </c>
       <c r="N83" s="22" t="s">
-        <v>983</v>
+        <v>977</v>
       </c>
       <c r="T83" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V83" s="22" t="s">
-        <v>900</v>
+        <v>894</v>
       </c>
       <c r="W83" s="24" t="s">
         <v>44</v>
@@ -10348,16 +10369,16 @@
         <v>81</v>
       </c>
       <c r="Z83" s="14" t="s">
-        <v>993</v>
+        <v>987</v>
       </c>
       <c r="AB83" s="22" t="s">
-        <v>902</v>
+        <v>896</v>
       </c>
       <c r="AC83" s="22" t="s">
-        <v>984</v>
+        <v>978</v>
       </c>
       <c r="AD83" s="23" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="84" spans="1:33" ht="45" x14ac:dyDescent="0.25">
@@ -10368,25 +10389,25 @@
         <v>33</v>
       </c>
       <c r="C84" s="7" t="s">
+        <v>658</v>
+      </c>
+      <c r="D84" s="16" t="s">
         <v>659</v>
       </c>
-      <c r="D84" s="16" t="s">
+      <c r="E84" s="16" t="s">
         <v>660</v>
-      </c>
-      <c r="E84" s="16" t="s">
-        <v>661</v>
       </c>
       <c r="F84" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I84" s="7" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="J84" s="7" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="L84" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M84" s="18" t="s">
         <v>51</v>
@@ -10404,13 +10425,13 @@
         <v>147</v>
       </c>
       <c r="AB84" s="22" t="s">
-        <v>899</v>
+        <v>893</v>
       </c>
       <c r="AC84" s="22" t="s">
-        <v>984</v>
+        <v>978</v>
       </c>
       <c r="AD84" s="23" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="85" spans="1:33" ht="45" x14ac:dyDescent="0.25">
@@ -10421,49 +10442,49 @@
         <v>33</v>
       </c>
       <c r="C85" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="D85" s="16" t="s">
         <v>663</v>
       </c>
-      <c r="D85" s="16" t="s">
+      <c r="E85" s="16" t="s">
         <v>664</v>
-      </c>
-      <c r="E85" s="16" t="s">
-        <v>665</v>
       </c>
       <c r="F85" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I85" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="J85" s="7" t="s">
         <v>666</v>
       </c>
-      <c r="J85" s="7" t="s">
+      <c r="K85" s="7" t="s">
         <v>667</v>
       </c>
-      <c r="K85" s="7" t="s">
+      <c r="L85" s="12" t="s">
+        <v>628</v>
+      </c>
+      <c r="M85" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="L85" s="12" t="s">
+      <c r="N85" s="18" t="s">
+        <v>669</v>
+      </c>
+      <c r="O85" s="16" t="s">
         <v>629</v>
       </c>
-      <c r="M85" s="18" t="s">
-        <v>669</v>
-      </c>
-      <c r="N85" s="18" t="s">
-        <v>670</v>
-      </c>
-      <c r="O85" s="16" t="s">
+      <c r="P85" s="16" t="s">
         <v>630</v>
-      </c>
-      <c r="P85" s="16" t="s">
-        <v>631</v>
       </c>
       <c r="S85" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T85" s="18" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="V85" s="22" t="s">
-        <v>901</v>
+        <v>895</v>
       </c>
       <c r="W85" s="16" t="s">
         <v>44</v>
@@ -10475,10 +10496,10 @@
         <v>92</v>
       </c>
       <c r="Z85" s="14" t="s">
-        <v>904</v>
+        <v>898</v>
       </c>
       <c r="AB85" s="22" t="s">
-        <v>902</v>
+        <v>896</v>
       </c>
     </row>
     <row r="86" spans="1:33" ht="375" x14ac:dyDescent="0.25">
@@ -10489,13 +10510,13 @@
         <v>33</v>
       </c>
       <c r="C86" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="D86" s="19" t="s">
         <v>671</v>
       </c>
-      <c r="D86" s="19" t="s">
+      <c r="E86" s="19" t="s">
         <v>672</v>
-      </c>
-      <c r="E86" s="19" t="s">
-        <v>673</v>
       </c>
       <c r="F86" s="13" t="s">
         <v>63</v>
@@ -10503,36 +10524,36 @@
       <c r="G86" s="13"/>
       <c r="H86" s="13"/>
       <c r="I86" s="13" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="J86" s="13" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="K86" s="13"/>
       <c r="L86" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M86" s="28" t="s">
+        <v>674</v>
+      </c>
+      <c r="N86" s="22" t="s">
+        <v>669</v>
+      </c>
+      <c r="O86" s="19" t="s">
         <v>675</v>
       </c>
-      <c r="N86" s="22" t="s">
-        <v>670</v>
-      </c>
-      <c r="O86" s="19" t="s">
+      <c r="P86" s="19" t="s">
         <v>676</v>
-      </c>
-      <c r="P86" s="19" t="s">
-        <v>677</v>
       </c>
       <c r="Q86" s="19"/>
       <c r="R86" s="30" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="S86" s="19" t="s">
         <v>43</v>
       </c>
       <c r="T86" s="29" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="U86" s="19"/>
       <c r="V86" s="28"/>
@@ -10546,14 +10567,14 @@
         <v>81</v>
       </c>
       <c r="Z86" s="14" t="s">
-        <v>909</v>
+        <v>903</v>
       </c>
       <c r="AA86" s="28" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="AB86" s="28"/>
       <c r="AC86" s="14" t="s">
-        <v>910</v>
+        <v>904</v>
       </c>
       <c r="AD86" s="28"/>
       <c r="AE86" s="19"/>
@@ -10568,37 +10589,37 @@
         <v>33</v>
       </c>
       <c r="C87" s="7" t="s">
+        <v>679</v>
+      </c>
+      <c r="D87" s="16" t="s">
         <v>680</v>
       </c>
-      <c r="D87" s="16" t="s">
+      <c r="E87" s="16" t="s">
         <v>681</v>
-      </c>
-      <c r="E87" s="16" t="s">
-        <v>682</v>
       </c>
       <c r="F87" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I87" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="J87" s="7" t="s">
         <v>683</v>
       </c>
-      <c r="J87" s="7" t="s">
-        <v>684</v>
-      </c>
       <c r="L87" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M87" s="22" t="s">
-        <v>914</v>
+        <v>908</v>
       </c>
       <c r="N87" s="22" t="s">
-        <v>915</v>
+        <v>909</v>
       </c>
       <c r="T87" s="22" t="s">
-        <v>916</v>
+        <v>910</v>
       </c>
       <c r="V87" s="22" t="s">
-        <v>917</v>
+        <v>911</v>
       </c>
       <c r="W87" s="24" t="s">
         <v>44</v>
@@ -10610,11 +10631,11 @@
         <v>81</v>
       </c>
       <c r="Z87" s="14" t="s">
-        <v>918</v>
+        <v>912</v>
       </c>
       <c r="AB87" s="28"/>
       <c r="AC87" s="22" t="s">
-        <v>919</v>
+        <v>913</v>
       </c>
     </row>
     <row r="88" spans="1:33" ht="60" x14ac:dyDescent="0.25">
@@ -10625,46 +10646,46 @@
         <v>33</v>
       </c>
       <c r="C88" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="D88" s="16" t="s">
         <v>685</v>
       </c>
-      <c r="D88" s="16" t="s">
+      <c r="E88" s="16" t="s">
         <v>686</v>
-      </c>
-      <c r="E88" s="16" t="s">
-        <v>687</v>
       </c>
       <c r="F88" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I88" s="7" t="s">
+        <v>687</v>
+      </c>
+      <c r="J88" s="7" t="s">
+        <v>683</v>
+      </c>
+      <c r="K88" s="7" t="s">
         <v>688</v>
       </c>
-      <c r="J88" s="7" t="s">
-        <v>684</v>
-      </c>
-      <c r="K88" s="7" t="s">
+      <c r="L88" s="12" t="s">
+        <v>628</v>
+      </c>
+      <c r="M88" s="18" t="s">
         <v>689</v>
       </c>
-      <c r="L88" s="12" t="s">
+      <c r="N88" s="18" t="s">
+        <v>690</v>
+      </c>
+      <c r="O88" s="16" t="s">
         <v>629</v>
       </c>
-      <c r="M88" s="18" t="s">
-        <v>690</v>
-      </c>
-      <c r="N88" s="18" t="s">
+      <c r="P88" s="16" t="s">
         <v>691</v>
-      </c>
-      <c r="O88" s="16" t="s">
-        <v>630</v>
-      </c>
-      <c r="P88" s="16" t="s">
-        <v>692</v>
       </c>
       <c r="S88" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T88" s="21" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="W88" s="16" t="s">
         <v>44</v>
@@ -10676,7 +10697,7 @@
         <v>92</v>
       </c>
       <c r="Z88" s="20" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="89" spans="1:33" ht="45" x14ac:dyDescent="0.25">
@@ -10687,22 +10708,22 @@
         <v>33</v>
       </c>
       <c r="C89" s="7" t="s">
+        <v>692</v>
+      </c>
+      <c r="D89" s="16" t="s">
         <v>693</v>
       </c>
-      <c r="D89" s="16" t="s">
-        <v>694</v>
-      </c>
       <c r="E89" s="16" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="F89" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K89" s="7" t="s">
+        <v>694</v>
+      </c>
+      <c r="L89" s="12" t="s">
         <v>695</v>
-      </c>
-      <c r="L89" s="12" t="s">
-        <v>696</v>
       </c>
       <c r="M89" s="18" t="s">
         <v>51</v>
@@ -10728,46 +10749,46 @@
         <v>33</v>
       </c>
       <c r="C90" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="D90" s="16" t="s">
         <v>697</v>
       </c>
-      <c r="D90" s="16" t="s">
+      <c r="E90" s="16" t="s">
         <v>698</v>
-      </c>
-      <c r="E90" s="16" t="s">
-        <v>699</v>
       </c>
       <c r="F90" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J90" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="K90" s="7" t="s">
         <v>700</v>
       </c>
-      <c r="K90" s="7" t="s">
+      <c r="L90" s="12" t="s">
+        <v>628</v>
+      </c>
+      <c r="M90" s="18" t="s">
         <v>701</v>
       </c>
-      <c r="L90" s="12" t="s">
+      <c r="N90" s="18" t="s">
+        <v>702</v>
+      </c>
+      <c r="O90" s="16" t="s">
         <v>629</v>
       </c>
-      <c r="M90" s="18" t="s">
-        <v>702</v>
-      </c>
-      <c r="N90" s="18" t="s">
+      <c r="P90" s="16" t="s">
         <v>703</v>
-      </c>
-      <c r="O90" s="16" t="s">
-        <v>630</v>
-      </c>
-      <c r="P90" s="16" t="s">
-        <v>704</v>
       </c>
       <c r="S90" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T90" s="18" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="V90" s="22" t="s">
-        <v>901</v>
+        <v>895</v>
       </c>
       <c r="W90" s="16" t="s">
         <v>44</v>
@@ -10778,14 +10799,14 @@
       <c r="Y90" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="Z90" s="20" t="s">
-        <v>654</v>
+      <c r="Z90" s="14" t="s">
+        <v>990</v>
       </c>
       <c r="AA90" s="18" t="s">
-        <v>705</v>
-      </c>
-      <c r="AC90" s="18" t="s">
-        <v>888</v>
+        <v>704</v>
+      </c>
+      <c r="AC90" s="22" t="s">
+        <v>989</v>
       </c>
     </row>
     <row r="91" spans="1:33" ht="75" x14ac:dyDescent="0.25">
@@ -10796,34 +10817,34 @@
         <v>33</v>
       </c>
       <c r="C91" s="7" t="s">
+        <v>705</v>
+      </c>
+      <c r="D91" s="16" t="s">
         <v>706</v>
       </c>
-      <c r="D91" s="16" t="s">
+      <c r="E91" s="16" t="s">
         <v>707</v>
-      </c>
-      <c r="E91" s="16" t="s">
-        <v>708</v>
       </c>
       <c r="F91" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J91" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L91" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M91" s="22" t="s">
-        <v>921</v>
+        <v>915</v>
       </c>
       <c r="N91" s="22" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="T91" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V91" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W91" s="24" t="s">
         <v>44</v>
@@ -10835,7 +10856,7 @@
         <v>81</v>
       </c>
       <c r="Z91" s="14" t="s">
-        <v>957</v>
+        <v>951</v>
       </c>
     </row>
     <row r="92" spans="1:33" ht="75" x14ac:dyDescent="0.25">
@@ -10846,34 +10867,34 @@
         <v>33</v>
       </c>
       <c r="C92" s="7" t="s">
+        <v>709</v>
+      </c>
+      <c r="D92" s="16" t="s">
         <v>710</v>
       </c>
-      <c r="D92" s="16" t="s">
+      <c r="E92" s="16" t="s">
         <v>711</v>
-      </c>
-      <c r="E92" s="16" t="s">
-        <v>712</v>
       </c>
       <c r="F92" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J92" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L92" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M92" s="22" t="s">
-        <v>922</v>
+        <v>916</v>
       </c>
       <c r="N92" s="22" t="s">
-        <v>935</v>
+        <v>929</v>
       </c>
       <c r="T92" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V92" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W92" s="24" t="s">
         <v>44</v>
@@ -10885,7 +10906,7 @@
         <v>81</v>
       </c>
       <c r="Z92" s="14" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
     </row>
     <row r="93" spans="1:33" ht="75" x14ac:dyDescent="0.25">
@@ -10896,34 +10917,34 @@
         <v>33</v>
       </c>
       <c r="C93" s="7" t="s">
+        <v>712</v>
+      </c>
+      <c r="D93" s="16" t="s">
         <v>713</v>
       </c>
-      <c r="D93" s="16" t="s">
+      <c r="E93" s="16" t="s">
         <v>714</v>
-      </c>
-      <c r="E93" s="16" t="s">
-        <v>715</v>
       </c>
       <c r="F93" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J93" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L93" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M93" s="22" t="s">
-        <v>923</v>
+        <v>917</v>
       </c>
       <c r="N93" s="22" t="s">
-        <v>936</v>
+        <v>930</v>
       </c>
       <c r="T93" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V93" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W93" s="24" t="s">
         <v>44</v>
@@ -10935,7 +10956,7 @@
         <v>81</v>
       </c>
       <c r="Z93" s="14" t="s">
-        <v>959</v>
+        <v>953</v>
       </c>
     </row>
     <row r="94" spans="1:33" ht="75" x14ac:dyDescent="0.25">
@@ -10946,34 +10967,34 @@
         <v>33</v>
       </c>
       <c r="C94" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="D94" s="16" t="s">
         <v>716</v>
       </c>
-      <c r="D94" s="16" t="s">
+      <c r="E94" s="16" t="s">
         <v>717</v>
-      </c>
-      <c r="E94" s="16" t="s">
-        <v>718</v>
       </c>
       <c r="F94" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J94" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L94" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M94" s="22" t="s">
-        <v>924</v>
+        <v>918</v>
       </c>
       <c r="N94" s="22" t="s">
-        <v>937</v>
+        <v>931</v>
       </c>
       <c r="T94" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V94" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W94" s="24" t="s">
         <v>44</v>
@@ -10985,7 +11006,7 @@
         <v>81</v>
       </c>
       <c r="Z94" s="14" t="s">
-        <v>960</v>
+        <v>954</v>
       </c>
     </row>
     <row r="95" spans="1:33" ht="45" x14ac:dyDescent="0.25">
@@ -10996,22 +11017,22 @@
         <v>33</v>
       </c>
       <c r="C95" s="7" t="s">
+        <v>718</v>
+      </c>
+      <c r="D95" s="16" t="s">
         <v>719</v>
       </c>
-      <c r="D95" s="16" t="s">
+      <c r="E95" s="16" t="s">
         <v>720</v>
-      </c>
-      <c r="E95" s="16" t="s">
-        <v>721</v>
       </c>
       <c r="F95" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J95" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L95" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M95" s="18" t="s">
         <v>51</v>
@@ -11037,34 +11058,34 @@
         <v>33</v>
       </c>
       <c r="C96" s="7" t="s">
+        <v>721</v>
+      </c>
+      <c r="D96" s="16" t="s">
         <v>722</v>
       </c>
-      <c r="D96" s="16" t="s">
+      <c r="E96" s="16" t="s">
         <v>723</v>
-      </c>
-      <c r="E96" s="16" t="s">
-        <v>724</v>
       </c>
       <c r="F96" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J96" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L96" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M96" s="22" t="s">
-        <v>925</v>
+        <v>919</v>
       </c>
       <c r="N96" s="22" t="s">
-        <v>938</v>
+        <v>932</v>
       </c>
       <c r="T96" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V96" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W96" s="24" t="s">
         <v>44</v>
@@ -11076,7 +11097,7 @@
         <v>81</v>
       </c>
       <c r="Z96" s="14" t="s">
-        <v>961</v>
+        <v>955</v>
       </c>
     </row>
     <row r="97" spans="1:26" ht="75" x14ac:dyDescent="0.25">
@@ -11087,34 +11108,34 @@
         <v>33</v>
       </c>
       <c r="C97" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="D97" s="16" t="s">
         <v>725</v>
       </c>
-      <c r="D97" s="16" t="s">
+      <c r="E97" s="16" t="s">
         <v>726</v>
-      </c>
-      <c r="E97" s="16" t="s">
-        <v>727</v>
       </c>
       <c r="F97" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J97" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L97" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M97" s="22" t="s">
-        <v>926</v>
+        <v>920</v>
       </c>
       <c r="N97" s="22" t="s">
-        <v>939</v>
+        <v>933</v>
       </c>
       <c r="T97" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V97" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W97" s="24" t="s">
         <v>44</v>
@@ -11126,7 +11147,7 @@
         <v>81</v>
       </c>
       <c r="Z97" s="14" t="s">
-        <v>962</v>
+        <v>956</v>
       </c>
     </row>
     <row r="98" spans="1:26" ht="75" x14ac:dyDescent="0.25">
@@ -11137,34 +11158,34 @@
         <v>33</v>
       </c>
       <c r="C98" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="D98" s="16" t="s">
         <v>728</v>
       </c>
-      <c r="D98" s="16" t="s">
+      <c r="E98" s="16" t="s">
         <v>729</v>
-      </c>
-      <c r="E98" s="16" t="s">
-        <v>730</v>
       </c>
       <c r="F98" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J98" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L98" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M98" s="22" t="s">
-        <v>927</v>
+        <v>921</v>
       </c>
       <c r="N98" s="22" t="s">
-        <v>940</v>
+        <v>934</v>
       </c>
       <c r="T98" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V98" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W98" s="24" t="s">
         <v>44</v>
@@ -11176,7 +11197,7 @@
         <v>81</v>
       </c>
       <c r="Z98" s="14" t="s">
-        <v>963</v>
+        <v>957</v>
       </c>
     </row>
     <row r="99" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11187,34 +11208,34 @@
         <v>33</v>
       </c>
       <c r="C99" s="7" t="s">
+        <v>730</v>
+      </c>
+      <c r="D99" s="16" t="s">
         <v>731</v>
       </c>
-      <c r="D99" s="16" t="s">
+      <c r="E99" s="16" t="s">
         <v>732</v>
-      </c>
-      <c r="E99" s="16" t="s">
-        <v>733</v>
       </c>
       <c r="F99" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J99" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L99" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M99" s="22" t="s">
-        <v>928</v>
+        <v>922</v>
       </c>
       <c r="N99" s="22" t="s">
-        <v>941</v>
+        <v>935</v>
       </c>
       <c r="T99" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V99" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W99" s="24" t="s">
         <v>44</v>
@@ -11226,7 +11247,7 @@
         <v>81</v>
       </c>
       <c r="Z99" s="14" t="s">
-        <v>964</v>
+        <v>958</v>
       </c>
     </row>
     <row r="100" spans="1:26" ht="75" x14ac:dyDescent="0.25">
@@ -11237,34 +11258,34 @@
         <v>33</v>
       </c>
       <c r="C100" s="7" t="s">
+        <v>733</v>
+      </c>
+      <c r="D100" s="16" t="s">
         <v>734</v>
       </c>
-      <c r="D100" s="16" t="s">
+      <c r="E100" s="16" t="s">
         <v>735</v>
-      </c>
-      <c r="E100" s="16" t="s">
-        <v>736</v>
       </c>
       <c r="F100" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J100" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L100" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M100" s="22" t="s">
-        <v>929</v>
+        <v>923</v>
       </c>
       <c r="N100" s="22" t="s">
-        <v>942</v>
+        <v>936</v>
       </c>
       <c r="T100" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V100" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W100" s="24" t="s">
         <v>44</v>
@@ -11276,7 +11297,7 @@
         <v>81</v>
       </c>
       <c r="Z100" s="14" t="s">
-        <v>965</v>
+        <v>959</v>
       </c>
     </row>
     <row r="101" spans="1:26" ht="75" x14ac:dyDescent="0.25">
@@ -11287,34 +11308,34 @@
         <v>33</v>
       </c>
       <c r="C101" s="7" t="s">
+        <v>736</v>
+      </c>
+      <c r="D101" s="16" t="s">
         <v>737</v>
       </c>
-      <c r="D101" s="16" t="s">
+      <c r="E101" s="16" t="s">
         <v>738</v>
-      </c>
-      <c r="E101" s="16" t="s">
-        <v>739</v>
       </c>
       <c r="F101" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J101" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L101" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M101" s="22" t="s">
-        <v>930</v>
+        <v>924</v>
       </c>
       <c r="N101" s="22" t="s">
-        <v>943</v>
+        <v>937</v>
       </c>
       <c r="T101" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V101" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W101" s="24" t="s">
         <v>44</v>
@@ -11326,7 +11347,7 @@
         <v>81</v>
       </c>
       <c r="Z101" s="14" t="s">
-        <v>966</v>
+        <v>960</v>
       </c>
     </row>
     <row r="102" spans="1:26" ht="75" x14ac:dyDescent="0.25">
@@ -11337,34 +11358,34 @@
         <v>33</v>
       </c>
       <c r="C102" s="7" t="s">
+        <v>739</v>
+      </c>
+      <c r="D102" s="16" t="s">
         <v>740</v>
       </c>
-      <c r="D102" s="16" t="s">
+      <c r="E102" s="16" t="s">
         <v>741</v>
-      </c>
-      <c r="E102" s="16" t="s">
-        <v>742</v>
       </c>
       <c r="F102" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J102" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L102" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M102" s="22" t="s">
-        <v>931</v>
+        <v>925</v>
       </c>
       <c r="N102" s="22" t="s">
-        <v>944</v>
+        <v>938</v>
       </c>
       <c r="T102" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V102" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W102" s="24" t="s">
         <v>44</v>
@@ -11376,7 +11397,7 @@
         <v>81</v>
       </c>
       <c r="Z102" s="14" t="s">
-        <v>967</v>
+        <v>961</v>
       </c>
     </row>
     <row r="103" spans="1:26" ht="75" x14ac:dyDescent="0.25">
@@ -11387,34 +11408,34 @@
         <v>33</v>
       </c>
       <c r="C103" s="7" t="s">
+        <v>742</v>
+      </c>
+      <c r="D103" s="16" t="s">
         <v>743</v>
       </c>
-      <c r="D103" s="16" t="s">
+      <c r="E103" s="16" t="s">
         <v>744</v>
-      </c>
-      <c r="E103" s="16" t="s">
-        <v>745</v>
       </c>
       <c r="F103" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J103" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L103" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M103" s="22" t="s">
-        <v>932</v>
+        <v>926</v>
       </c>
       <c r="N103" s="22" t="s">
-        <v>945</v>
+        <v>939</v>
       </c>
       <c r="T103" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V103" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W103" s="24" t="s">
         <v>44</v>
@@ -11426,7 +11447,7 @@
         <v>81</v>
       </c>
       <c r="Z103" s="14" t="s">
-        <v>968</v>
+        <v>962</v>
       </c>
     </row>
     <row r="104" spans="1:26" ht="75" x14ac:dyDescent="0.25">
@@ -11437,34 +11458,34 @@
         <v>33</v>
       </c>
       <c r="C104" s="7" t="s">
+        <v>745</v>
+      </c>
+      <c r="D104" s="16" t="s">
         <v>746</v>
       </c>
-      <c r="D104" s="16" t="s">
+      <c r="E104" s="16" t="s">
         <v>747</v>
-      </c>
-      <c r="E104" s="16" t="s">
-        <v>748</v>
       </c>
       <c r="F104" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J104" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L104" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M104" s="22" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="N104" s="22" t="s">
-        <v>946</v>
+        <v>940</v>
       </c>
       <c r="T104" s="22" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="V104" s="22" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="W104" s="24" t="s">
         <v>44</v>
@@ -11476,7 +11497,7 @@
         <v>81</v>
       </c>
       <c r="Z104" s="14" t="s">
-        <v>969</v>
+        <v>963</v>
       </c>
     </row>
     <row r="105" spans="1:26" ht="45" x14ac:dyDescent="0.25">
@@ -11487,22 +11508,22 @@
         <v>33</v>
       </c>
       <c r="C105" s="7" t="s">
+        <v>748</v>
+      </c>
+      <c r="D105" s="16" t="s">
         <v>749</v>
       </c>
-      <c r="D105" s="16" t="s">
+      <c r="E105" s="16" t="s">
         <v>750</v>
-      </c>
-      <c r="E105" s="16" t="s">
-        <v>751</v>
       </c>
       <c r="F105" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J105" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L105" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M105" s="18" t="s">
         <v>51</v>
@@ -11528,22 +11549,22 @@
         <v>33</v>
       </c>
       <c r="C106" s="7" t="s">
+        <v>751</v>
+      </c>
+      <c r="D106" s="16" t="s">
         <v>752</v>
       </c>
-      <c r="D106" s="16" t="s">
+      <c r="E106" s="16" t="s">
         <v>753</v>
-      </c>
-      <c r="E106" s="16" t="s">
-        <v>754</v>
       </c>
       <c r="F106" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J106" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L106" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M106" s="18" t="s">
         <v>51</v>
@@ -11569,22 +11590,22 @@
         <v>33</v>
       </c>
       <c r="C107" s="7" t="s">
+        <v>754</v>
+      </c>
+      <c r="D107" s="16" t="s">
         <v>755</v>
       </c>
-      <c r="D107" s="16" t="s">
+      <c r="E107" s="16" t="s">
         <v>756</v>
-      </c>
-      <c r="E107" s="16" t="s">
-        <v>757</v>
       </c>
       <c r="F107" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J107" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L107" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M107" s="18" t="s">
         <v>51</v>
@@ -11610,22 +11631,22 @@
         <v>33</v>
       </c>
       <c r="C108" s="7" t="s">
+        <v>757</v>
+      </c>
+      <c r="D108" s="16" t="s">
         <v>758</v>
       </c>
-      <c r="D108" s="16" t="s">
+      <c r="E108" s="16" t="s">
         <v>759</v>
-      </c>
-      <c r="E108" s="16" t="s">
-        <v>760</v>
       </c>
       <c r="F108" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J108" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L108" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M108" s="18" t="s">
         <v>51</v>
@@ -11651,22 +11672,22 @@
         <v>33</v>
       </c>
       <c r="C109" s="7" t="s">
+        <v>760</v>
+      </c>
+      <c r="D109" s="16" t="s">
         <v>761</v>
       </c>
-      <c r="D109" s="16" t="s">
+      <c r="E109" s="16" t="s">
         <v>762</v>
-      </c>
-      <c r="E109" s="16" t="s">
-        <v>763</v>
       </c>
       <c r="F109" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J109" s="7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L109" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M109" s="18" t="s">
         <v>51</v>
@@ -11692,22 +11713,22 @@
         <v>33</v>
       </c>
       <c r="C110" s="7" t="s">
+        <v>763</v>
+      </c>
+      <c r="D110" s="16" t="s">
         <v>764</v>
       </c>
-      <c r="D110" s="16" t="s">
+      <c r="E110" s="16" t="s">
         <v>765</v>
-      </c>
-      <c r="E110" s="16" t="s">
-        <v>766</v>
       </c>
       <c r="F110" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J110" s="7" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="L110" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M110" s="18" t="s">
         <v>51</v>
@@ -11733,22 +11754,22 @@
         <v>33</v>
       </c>
       <c r="C111" s="7" t="s">
+        <v>767</v>
+      </c>
+      <c r="D111" s="16" t="s">
         <v>768</v>
       </c>
-      <c r="D111" s="16" t="s">
+      <c r="E111" s="16" t="s">
         <v>769</v>
-      </c>
-      <c r="E111" s="16" t="s">
-        <v>770</v>
       </c>
       <c r="F111" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J111" s="7" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="L111" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M111" s="18" t="s">
         <v>51</v>
@@ -11774,22 +11795,22 @@
         <v>33</v>
       </c>
       <c r="C112" s="7" t="s">
+        <v>771</v>
+      </c>
+      <c r="D112" s="16" t="s">
         <v>772</v>
       </c>
-      <c r="D112" s="16" t="s">
+      <c r="E112" s="16" t="s">
         <v>773</v>
-      </c>
-      <c r="E112" s="16" t="s">
-        <v>774</v>
       </c>
       <c r="F112" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J112" s="7" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="L112" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M112" s="18" t="s">
         <v>51</v>
@@ -11815,28 +11836,28 @@
         <v>33</v>
       </c>
       <c r="C113" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="D113" s="16" t="s">
         <v>775</v>
       </c>
-      <c r="D113" s="16" t="s">
-        <v>776</v>
-      </c>
       <c r="E113" s="16" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="F113" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J113" s="7" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="L113" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M113" s="22" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
       <c r="N113" s="22" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
       <c r="O113" s="24"/>
       <c r="P113" s="24"/>
@@ -11844,10 +11865,10 @@
       <c r="R113" s="24"/>
       <c r="S113" s="24"/>
       <c r="T113" s="22" t="s">
-        <v>948</v>
+        <v>942</v>
       </c>
       <c r="V113" s="22" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
       <c r="W113" s="16" t="s">
         <v>44</v>
@@ -11859,16 +11880,16 @@
         <v>81</v>
       </c>
       <c r="Z113" s="14" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
       <c r="AA113" s="18" t="s">
+        <v>777</v>
+      </c>
+      <c r="AB113" s="27" t="s">
         <v>778</v>
       </c>
-      <c r="AB113" s="27" t="s">
-        <v>779</v>
-      </c>
       <c r="AC113" s="22" t="s">
-        <v>952</v>
+        <v>946</v>
       </c>
     </row>
     <row r="114" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
@@ -11879,28 +11900,28 @@
         <v>33</v>
       </c>
       <c r="C114" s="7" t="s">
+        <v>779</v>
+      </c>
+      <c r="D114" s="16" t="s">
         <v>780</v>
       </c>
-      <c r="D114" s="16" t="s">
-        <v>781</v>
-      </c>
       <c r="E114" s="16" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="F114" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J114" s="7" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="L114" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M114" s="22" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
       <c r="N114" s="22" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
       <c r="O114" s="24"/>
       <c r="P114" s="24"/>
@@ -11908,10 +11929,10 @@
       <c r="R114" s="24"/>
       <c r="S114" s="24"/>
       <c r="T114" s="22" t="s">
-        <v>948</v>
+        <v>942</v>
       </c>
       <c r="V114" s="22" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
       <c r="W114" s="16" t="s">
         <v>44</v>
@@ -11923,13 +11944,13 @@
         <v>81</v>
       </c>
       <c r="Z114" s="14" t="s">
-        <v>954</v>
+        <v>948</v>
       </c>
       <c r="AA114" s="18" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="AC114" s="22" t="s">
-        <v>952</v>
+        <v>946</v>
       </c>
     </row>
     <row r="115" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
@@ -11940,28 +11961,28 @@
         <v>33</v>
       </c>
       <c r="C115" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="D115" s="16" t="s">
         <v>784</v>
       </c>
-      <c r="D115" s="16" t="s">
-        <v>785</v>
-      </c>
       <c r="E115" s="16" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="F115" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J115" s="7" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="L115" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="M115" s="22" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
       <c r="N115" s="22" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
       <c r="O115" s="24"/>
       <c r="P115" s="24"/>
@@ -11969,10 +11990,10 @@
       <c r="R115" s="24"/>
       <c r="S115" s="24"/>
       <c r="T115" s="22" t="s">
-        <v>948</v>
+        <v>942</v>
       </c>
       <c r="V115" s="22" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
       <c r="W115" s="16" t="s">
         <v>44</v>
@@ -11984,16 +12005,16 @@
         <v>81</v>
       </c>
       <c r="Z115" s="14" t="s">
-        <v>955</v>
+        <v>949</v>
       </c>
       <c r="AA115" s="18" t="s">
+        <v>785</v>
+      </c>
+      <c r="AB115" s="18" t="s">
         <v>786</v>
       </c>
-      <c r="AB115" s="18" t="s">
-        <v>787</v>
-      </c>
       <c r="AC115" s="22" t="s">
-        <v>952</v>
+        <v>946</v>
       </c>
     </row>
     <row r="116" spans="1:29" x14ac:dyDescent="0.25">
@@ -12004,19 +12025,19 @@
         <v>33</v>
       </c>
       <c r="C116" s="7" t="s">
+        <v>787</v>
+      </c>
+      <c r="D116" s="16" t="s">
         <v>788</v>
       </c>
-      <c r="D116" s="16" t="s">
-        <v>789</v>
-      </c>
       <c r="E116" s="16" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="F116" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J116" s="7" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="M116" s="18" t="s">
         <v>51</v>
@@ -12042,19 +12063,19 @@
         <v>33</v>
       </c>
       <c r="C117" s="7" t="s">
+        <v>790</v>
+      </c>
+      <c r="D117" s="16" t="s">
         <v>791</v>
       </c>
-      <c r="D117" s="16" t="s">
-        <v>792</v>
-      </c>
       <c r="E117" s="16" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="F117" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J117" s="7" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="M117" s="18" t="s">
         <v>51</v>
@@ -12080,40 +12101,40 @@
         <v>33</v>
       </c>
       <c r="C118" s="7" t="s">
+        <v>793</v>
+      </c>
+      <c r="D118" s="16" t="s">
         <v>794</v>
       </c>
-      <c r="D118" s="16" t="s">
-        <v>795</v>
-      </c>
       <c r="E118" s="16" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="F118" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J118" s="7" t="s">
+        <v>795</v>
+      </c>
+      <c r="M118" s="18" t="s">
         <v>796</v>
       </c>
-      <c r="M118" s="18" t="s">
+      <c r="N118" s="18" t="s">
         <v>797</v>
       </c>
-      <c r="N118" s="18" t="s">
+      <c r="O118" s="16" t="s">
         <v>798</v>
       </c>
-      <c r="O118" s="16" t="s">
+      <c r="P118" s="16" t="s">
         <v>799</v>
       </c>
-      <c r="P118" s="16" t="s">
+      <c r="Q118" s="16" t="s">
         <v>800</v>
-      </c>
-      <c r="Q118" s="16" t="s">
-        <v>801</v>
       </c>
       <c r="S118" s="16" t="s">
         <v>104</v>
       </c>
       <c r="T118" s="18" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="W118" s="16" t="s">
         <v>44</v>
@@ -12125,10 +12146,10 @@
         <v>81</v>
       </c>
       <c r="Z118" s="14" t="s">
-        <v>947</v>
+        <v>941</v>
       </c>
       <c r="AC118" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="119" spans="1:29" x14ac:dyDescent="0.25">
@@ -12139,19 +12160,19 @@
         <v>33</v>
       </c>
       <c r="C119" s="7" t="s">
+        <v>802</v>
+      </c>
+      <c r="D119" s="16" t="s">
         <v>803</v>
       </c>
-      <c r="D119" s="16" t="s">
-        <v>804</v>
-      </c>
       <c r="E119" s="16" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="F119" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J119" s="7" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="M119" s="18" t="s">
         <v>51</v>
@@ -12177,22 +12198,22 @@
         <v>33</v>
       </c>
       <c r="C120" s="7" t="s">
+        <v>805</v>
+      </c>
+      <c r="D120" s="16" t="s">
         <v>806</v>
       </c>
-      <c r="D120" s="16" t="s">
-        <v>807</v>
-      </c>
       <c r="E120" s="16" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="F120" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J120" s="7" t="s">
+        <v>807</v>
+      </c>
+      <c r="K120" s="7" t="s">
         <v>808</v>
-      </c>
-      <c r="K120" s="7" t="s">
-        <v>809</v>
       </c>
       <c r="M120" s="18" t="s">
         <v>51</v>
@@ -12218,19 +12239,19 @@
         <v>33</v>
       </c>
       <c r="C121" s="7" t="s">
+        <v>809</v>
+      </c>
+      <c r="D121" s="16" t="s">
         <v>810</v>
       </c>
-      <c r="D121" s="16" t="s">
-        <v>811</v>
-      </c>
       <c r="E121" s="16" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="F121" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J121" s="7" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="M121" s="18" t="s">
         <v>51</v>
@@ -12256,19 +12277,19 @@
         <v>33</v>
       </c>
       <c r="C122" s="7" t="s">
+        <v>811</v>
+      </c>
+      <c r="D122" s="16" t="s">
         <v>812</v>
       </c>
-      <c r="D122" s="16" t="s">
-        <v>813</v>
-      </c>
       <c r="E122" s="16" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="F122" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J122" s="7" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="M122" s="18" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
Correct coding of Presumed no.
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-BCS.xlsx
+++ b/baseline/data_processing_elements-BCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E547C0-2627-4353-856E-DD00455C7286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4CE1C12-BE95-46B3-9DCA-6234A9CF88E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="1840" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
@@ -3988,20 +3988,11 @@
     <t>Would "irregular heartbeat" be considered atrial fibrillation?</t>
   </si>
   <si>
-    <t>The study-specific variable asks about types of heart problems since last interview/4 years.</t>
-  </si>
-  <si>
-    <t>The study-specific variable asks about types of health problems since last interview/4 years.</t>
-  </si>
-  <si>
     <t>Variables are not in "ever" format. In general, how should these types of variable be handled?</t>
   </si>
   <si>
     <t>Should variable BD10SYMPAN1 from Rose Qx be incorporated?
 Category -1 Not applicable is No.</t>
-  </si>
-  <si>
-    <t>recode(0 = 0 ; 1 = 1 ; -8 = NA ; ELSE = NA)</t>
   </si>
   <si>
     <t>Health probs since last int/4 yrs ago: High blood pressure;
@@ -4063,10 +4054,6 @@
 (-9) Refused   (-8) Not known   (-1) Not applicable    (0) No    (1) Yes </t>
   </si>
   <si>
-    <t>The study-specific variables ask about types of health or back problems since last interview/4 years. 
-Arthritis reported under health problems or back problems coded as 1=Yes. Could not assign 0=No.</t>
-  </si>
-  <si>
     <t>case_when(
 B10KHPB19 == 1 | B10BCKP50 == 1 ~ 1L ; 
 ELSE ~ NA_integer_)</t>
@@ -4074,10 +4061,6 @@
   <si>
     <t>Have variable for arthritis. Could assign 1. 
 There is a section about Musculoskeletal system, but only questions about back problems.</t>
-  </si>
-  <si>
-    <t>The study-specific variable asks about types of heart problems since last interview/4 years. 
-Only self-reported responses are used. A study-specific variable based on score from the Rose Questionnaire is not used.</t>
   </si>
   <si>
     <t>B10CCTY50 ; 
@@ -4505,100 +4488,6 @@
 ELSE ~ 0L)</t>
   </si>
   <si>
-    <t>The study-specific variable asks about types of cancer since last interview/4 years.</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY50 == 1 ~ 1L ; 
-B10CCTY50 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY06 == 1 ~ 1L ; 
-B10CCTY06 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY08 == 1 ~ 1L ; 
-B10CCTY08 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY11 == 1 ~ 1L ; 
-B10CCTY11 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY51 == 1 ~ 1L ; 
-B10CCTY51 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY01 == 1 ~ 1L ; 
-B10CCTY01 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY13 == 1 ~ 1L ; 
-B10CCTY13 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY02 == 1 | B10CCTY03 == 1 ~ 1L ; 
-B10CCTY02 == 0 &amp; B10CCTY03 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY10 == 1 ~ 1L ; 
-B10CCTY10 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY04 == 1 ~ 1L ; 
-B10CCTY04 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY12 == 1 ~ 1L ; 
-B10CCTY12 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY09 == 1 ~ 1L ; 
-B10CCTY09 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10CCTY07 == 1 ~ 1L ; 
-B10CCTY07 == 0 ~ 0L ; 
-B10KHPB06 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
     <t>Already integer. Changed to direct_mapping. 
 Range 45-48.</t>
   </si>
@@ -4677,44 +4566,7 @@
 B10KHPB11</t>
   </si>
   <si>
-    <t>case_when(
-B10HRTP02 == 1 ~ 1L ; 
-B10HRTP02 == 0 ~ 0L ; 
-B10KHPB11 == 0 ~ 0L ;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10HRTP01 == 1 ~ 1L ; 
-B10HRTP01 == 0 ~ 0L ; 
-B10KHPB11 == 0 ~ 0L ;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10HRTP03 == 1 ~ 1L ; 
-B10HRTP03 == 0 ~ 0L ; 
-B10KHPB11 == 0 ~ 0L ;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-B10HRTP04 == 1 ~ 1L ; 
-B10HRTP04 == 0 ~ 0L ; 
-B10KHPB11 == 0 ~ 0L ;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
     <t>Only one population.</t>
-  </si>
-  <si>
-    <t>Changed to code No.</t>
-  </si>
-  <si>
-    <t>recode(
-0=0;
-1=1;
-ELSE=NA)</t>
   </si>
   <si>
     <t>Add condition "Leave missing when triglycerides exceed 4.5 mmol/L (400 mg/dL)."</t>
@@ -4753,6 +4605,156 @@
     <t>case_when(
 B10WAISTAV &gt; 0 ~ as.numeric(B10WAISTAV) ; 
 ELSE ~ NA_real_)</t>
+  </si>
+  <si>
+    <t>Categories are Yes/No. Changed to code No.</t>
+  </si>
+  <si>
+    <t>case_when(
+B10HRTP02 == 1 ~ 1L ; 
+B10HRTP02 == 0 ~ 2L ; 
+B10KHPB11 == 0 ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10HRTP01 == 1 ~ 1L ; 
+B10HRTP01 == 0 ~ 2L ; 
+B10KHPB11 == 0 ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10HRTP03 == 1 ~ 1L ; 
+B10HRTP03 == 0 ~ 2L ; 
+B10KHPB11 == 0 ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>recode(0 = 2 ; 1 = 1 ; -8 = NA ; ELSE = NA)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10HRTP04 == 1 ~ 1L ; 
+B10HRTP04 == 0 ~ 2L ; 
+B10KHPB11 == 0 ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY50 == 1 ~ 1L ; 
+B10CCTY50 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY06 == 1 ~ 1L ; 
+B10CCTY06 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY08 == 1 ~ 1L ; 
+B10CCTY08 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY11 == 1 ~ 1L ; 
+B10CCTY11 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY51 == 1 ~ 1L ; 
+B10CCTY51 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY01 == 1 ~ 1L ; 
+B10CCTY01 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY13 == 1 ~ 1L ; 
+B10CCTY13 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY02 == 1 | B10CCTY03 == 1 ~ 1L ; 
+B10CCTY02 == 0 &amp; B10CCTY03 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY10 == 1 ~ 1L ; 
+B10CCTY10 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY04 == 1 ~ 1L ; 
+B10CCTY04 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY12 == 1 ~ 1L ; 
+B10CCTY12 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY09 == 1 ~ 1L ; 
+B10CCTY09 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+B10CCTY07 == 1 ~ 1L ; 
+B10CCTY07 == 0 ~ 2L ; 
+B10KHPB06 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>The study-specific variables ask about types of health problems since last interview/4 years.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
+  </si>
+  <si>
+    <t>The study-specific variable asks about types of heart problems since last interview/4 years.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
+  </si>
+  <si>
+    <t>The study-specific variable asks about types of heart problems since last interview/4 years. 
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.
+Only self-reported responses are used. A study-specific variable based on score from the Rose Questionnaire is not used.</t>
+  </si>
+  <si>
+    <t>The study-specific variable asks about types of health problems since last interview/4 years.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
+  </si>
+  <si>
+    <t>The study-specific variables ask about types of health or back problems since last interview/4 years. 
+Arthritis reported under health problems or back problems coded as 1=Yes. Could not assign Presumed no.</t>
+  </si>
+  <si>
+    <t>The study-specific variable asks about types of cancer since last interview/4 years.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
   </si>
 </sst>
 </file>
@@ -5569,7 +5571,7 @@
         <v>59</v>
       </c>
       <c r="AC4" s="22" t="s">
-        <v>988</v>
+        <v>965</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -5793,7 +5795,7 @@
         <v>848</v>
       </c>
       <c r="AC8" s="18" t="s">
-        <v>964</v>
+        <v>945</v>
       </c>
     </row>
     <row r="9" spans="1:33" ht="180" x14ac:dyDescent="0.25">
@@ -7388,7 +7390,7 @@
         <v>81</v>
       </c>
       <c r="Z32" s="14" t="s">
-        <v>998</v>
+        <v>973</v>
       </c>
       <c r="AC32" s="22" t="s">
         <v>858</v>
@@ -7506,13 +7508,13 @@
         <v>81</v>
       </c>
       <c r="Z34" s="14" t="s">
-        <v>996</v>
+        <v>971</v>
       </c>
       <c r="AA34" s="18" t="s">
         <v>315</v>
       </c>
       <c r="AC34" s="22" t="s">
-        <v>997</v>
+        <v>972</v>
       </c>
     </row>
     <row r="35" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8229,13 +8231,13 @@
         <v>81</v>
       </c>
       <c r="Z46" s="14" t="s">
-        <v>992</v>
+        <v>967</v>
       </c>
       <c r="AA46" s="18" t="s">
         <v>409</v>
       </c>
       <c r="AC46" s="22" t="s">
-        <v>991</v>
+        <v>966</v>
       </c>
     </row>
     <row r="47" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8727,7 +8729,7 @@
         <v>884</v>
       </c>
       <c r="AC55" s="27" t="s">
-        <v>965</v>
+        <v>946</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="120" x14ac:dyDescent="0.25">
@@ -8848,7 +8850,7 @@
         <v>92</v>
       </c>
       <c r="Z57" s="14" t="s">
-        <v>966</v>
+        <v>947</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="75" x14ac:dyDescent="0.25">
@@ -8910,7 +8912,7 @@
         <v>81</v>
       </c>
       <c r="Z58" s="22" t="s">
-        <v>967</v>
+        <v>948</v>
       </c>
       <c r="AA58" s="18" t="s">
         <v>455</v>
@@ -8969,7 +8971,7 @@
         <v>81</v>
       </c>
       <c r="Z59" s="20" t="s">
-        <v>968</v>
+        <v>949</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="195" x14ac:dyDescent="0.25">
@@ -9129,7 +9131,7 @@
         <v>513</v>
       </c>
       <c r="V62" s="22" t="s">
-        <v>993</v>
+        <v>968</v>
       </c>
       <c r="W62" s="16" t="s">
         <v>44</v>
@@ -9144,7 +9146,7 @@
         <v>514</v>
       </c>
       <c r="AC62" s="22" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
     </row>
     <row r="63" spans="1:31" ht="135" x14ac:dyDescent="0.25">
@@ -9341,7 +9343,7 @@
         <v>520</v>
       </c>
       <c r="V66" s="22" t="s">
-        <v>994</v>
+        <v>969</v>
       </c>
       <c r="W66" s="16" t="s">
         <v>44</v>
@@ -9356,7 +9358,7 @@
         <v>538</v>
       </c>
       <c r="AC66" s="22" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
     </row>
     <row r="67" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -9403,7 +9405,7 @@
         <v>513</v>
       </c>
       <c r="V67" s="22" t="s">
-        <v>995</v>
+        <v>970</v>
       </c>
       <c r="W67" s="16" t="s">
         <v>44</v>
@@ -9418,7 +9420,7 @@
         <v>546</v>
       </c>
       <c r="AC67" s="22" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
     </row>
     <row r="68" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -9556,7 +9558,7 @@
         <v>562</v>
       </c>
       <c r="V70" s="22" t="s">
-        <v>969</v>
+        <v>950</v>
       </c>
       <c r="W70" s="16" t="s">
         <v>44</v>
@@ -9571,7 +9573,7 @@
         <v>563</v>
       </c>
       <c r="AC70" s="22" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
     </row>
     <row r="71" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -9630,7 +9632,7 @@
         <v>573</v>
       </c>
       <c r="AC71" s="22" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
     </row>
     <row r="72" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -9695,7 +9697,7 @@
         <v>581</v>
       </c>
       <c r="AC72" s="22" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
     </row>
     <row r="73" spans="1:30" ht="135" x14ac:dyDescent="0.25">
@@ -9742,7 +9744,7 @@
         <v>590</v>
       </c>
       <c r="V73" s="27" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="W73" s="16" t="s">
         <v>44</v>
@@ -9757,7 +9759,7 @@
         <v>591</v>
       </c>
       <c r="AC73" s="27" t="s">
-        <v>907</v>
+        <v>904</v>
       </c>
     </row>
     <row r="74" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -9822,7 +9824,7 @@
         <v>598</v>
       </c>
       <c r="AC74" s="22" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
     </row>
     <row r="75" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -9848,10 +9850,10 @@
         <v>602</v>
       </c>
       <c r="M75" s="22" t="s">
-        <v>970</v>
+        <v>951</v>
       </c>
       <c r="N75" s="22" t="s">
-        <v>971</v>
+        <v>952</v>
       </c>
       <c r="O75" s="24" t="s">
         <v>605</v>
@@ -9865,7 +9867,7 @@
         <v>43</v>
       </c>
       <c r="T75" s="33" t="s">
-        <v>973</v>
+        <v>954</v>
       </c>
       <c r="W75" s="32" t="s">
         <v>44</v>
@@ -9877,13 +9879,13 @@
         <v>81</v>
       </c>
       <c r="Z75" s="14" t="s">
-        <v>974</v>
+        <v>955</v>
       </c>
       <c r="AA75" s="22" t="s">
         <v>608</v>
       </c>
       <c r="AC75" s="22" t="s">
-        <v>972</v>
+        <v>953</v>
       </c>
     </row>
     <row r="76" spans="1:30" ht="225" x14ac:dyDescent="0.25">
@@ -10027,10 +10029,10 @@
         <v>628</v>
       </c>
       <c r="M78" s="22" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
       <c r="N78" s="22" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="O78" s="24" t="s">
         <v>629</v>
@@ -10047,7 +10049,7 @@
         <v>631</v>
       </c>
       <c r="V78" s="22" t="s">
-        <v>895</v>
+        <v>993</v>
       </c>
       <c r="W78" s="16" t="s">
         <v>44</v>
@@ -10059,13 +10061,13 @@
         <v>81</v>
       </c>
       <c r="Z78" s="14" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="AC78" s="22" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
     </row>
-    <row r="79" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" ht="90" x14ac:dyDescent="0.25">
       <c r="A79" s="17">
         <v>78</v>
       </c>
@@ -10094,16 +10096,16 @@
         <v>628</v>
       </c>
       <c r="M79" s="22" t="s">
-        <v>980</v>
+        <v>961</v>
       </c>
       <c r="N79" s="22" t="s">
-        <v>975</v>
+        <v>956</v>
       </c>
       <c r="T79" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V79" s="22" t="s">
-        <v>894</v>
+        <v>994</v>
       </c>
       <c r="W79" s="24" t="s">
         <v>44</v>
@@ -10115,16 +10117,16 @@
         <v>81</v>
       </c>
       <c r="Z79" s="14" t="s">
-        <v>984</v>
+        <v>975</v>
       </c>
       <c r="AB79" s="22" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="AD79" s="23" t="s">
         <v>824</v>
       </c>
     </row>
-    <row r="80" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:30" ht="90" x14ac:dyDescent="0.25">
       <c r="A80" s="17">
         <v>79</v>
       </c>
@@ -10153,16 +10155,16 @@
         <v>628</v>
       </c>
       <c r="M80" s="22" t="s">
-        <v>981</v>
+        <v>962</v>
       </c>
       <c r="N80" s="22" t="s">
-        <v>976</v>
+        <v>957</v>
       </c>
       <c r="T80" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V80" s="22" t="s">
-        <v>894</v>
+        <v>994</v>
       </c>
       <c r="W80" s="24" t="s">
         <v>44</v>
@@ -10174,19 +10176,19 @@
         <v>81</v>
       </c>
       <c r="Z80" s="14" t="s">
-        <v>985</v>
+        <v>976</v>
       </c>
       <c r="AB80" s="22" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="AC80" s="22" t="s">
-        <v>978</v>
+        <v>959</v>
       </c>
       <c r="AD80" s="23" t="s">
         <v>824</v>
       </c>
     </row>
-    <row r="81" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:33" ht="135" x14ac:dyDescent="0.25">
       <c r="A81" s="17">
         <v>80</v>
       </c>
@@ -10215,16 +10217,16 @@
         <v>628</v>
       </c>
       <c r="M81" s="22" t="s">
-        <v>982</v>
+        <v>963</v>
       </c>
       <c r="N81" s="22" t="s">
-        <v>979</v>
+        <v>960</v>
       </c>
       <c r="T81" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V81" s="22" t="s">
-        <v>914</v>
+        <v>995</v>
       </c>
       <c r="W81" s="24" t="s">
         <v>44</v>
@@ -10236,19 +10238,19 @@
         <v>81</v>
       </c>
       <c r="Z81" s="14" t="s">
-        <v>986</v>
+        <v>977</v>
       </c>
       <c r="AB81" s="22" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="AC81" s="27" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="AD81" s="23" t="s">
         <v>824</v>
       </c>
     </row>
-    <row r="82" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A82" s="17">
         <v>81</v>
       </c>
@@ -10295,7 +10297,7 @@
         <v>652</v>
       </c>
       <c r="V82" s="22" t="s">
-        <v>895</v>
+        <v>996</v>
       </c>
       <c r="W82" s="16" t="s">
         <v>44</v>
@@ -10307,19 +10309,19 @@
         <v>92</v>
       </c>
       <c r="Z82" s="14" t="s">
-        <v>898</v>
+        <v>978</v>
       </c>
       <c r="AB82" s="22" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="AC82" s="22" t="s">
-        <v>978</v>
+        <v>959</v>
       </c>
       <c r="AD82" s="23" t="s">
         <v>824</v>
       </c>
     </row>
-    <row r="83" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A83" s="17">
         <v>82</v>
       </c>
@@ -10348,16 +10350,16 @@
         <v>628</v>
       </c>
       <c r="M83" s="22" t="s">
-        <v>983</v>
+        <v>964</v>
       </c>
       <c r="N83" s="22" t="s">
-        <v>977</v>
+        <v>958</v>
       </c>
       <c r="T83" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V83" s="22" t="s">
-        <v>894</v>
+        <v>994</v>
       </c>
       <c r="W83" s="24" t="s">
         <v>44</v>
@@ -10369,13 +10371,13 @@
         <v>81</v>
       </c>
       <c r="Z83" s="14" t="s">
-        <v>987</v>
+        <v>979</v>
       </c>
       <c r="AB83" s="22" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="AC83" s="22" t="s">
-        <v>978</v>
+        <v>959</v>
       </c>
       <c r="AD83" s="23" t="s">
         <v>824</v>
@@ -10428,13 +10430,13 @@
         <v>893</v>
       </c>
       <c r="AC84" s="22" t="s">
-        <v>978</v>
+        <v>959</v>
       </c>
       <c r="AD84" s="23" t="s">
         <v>825</v>
       </c>
     </row>
-    <row r="85" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A85" s="17">
         <v>84</v>
       </c>
@@ -10484,7 +10486,7 @@
         <v>652</v>
       </c>
       <c r="V85" s="22" t="s">
-        <v>895</v>
+        <v>996</v>
       </c>
       <c r="W85" s="16" t="s">
         <v>44</v>
@@ -10496,10 +10498,10 @@
         <v>92</v>
       </c>
       <c r="Z85" s="14" t="s">
-        <v>898</v>
+        <v>978</v>
       </c>
       <c r="AB85" s="22" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
     </row>
     <row r="86" spans="1:33" ht="375" x14ac:dyDescent="0.25">
@@ -10567,14 +10569,14 @@
         <v>81</v>
       </c>
       <c r="Z86" s="14" t="s">
-        <v>903</v>
+        <v>900</v>
       </c>
       <c r="AA86" s="28" t="s">
         <v>455</v>
       </c>
       <c r="AB86" s="28"/>
       <c r="AC86" s="14" t="s">
-        <v>904</v>
+        <v>901</v>
       </c>
       <c r="AD86" s="28"/>
       <c r="AE86" s="19"/>
@@ -10610,16 +10612,16 @@
         <v>628</v>
       </c>
       <c r="M87" s="22" t="s">
-        <v>908</v>
+        <v>905</v>
       </c>
       <c r="N87" s="22" t="s">
-        <v>909</v>
+        <v>906</v>
       </c>
       <c r="T87" s="22" t="s">
-        <v>910</v>
+        <v>907</v>
       </c>
       <c r="V87" s="22" t="s">
-        <v>911</v>
+        <v>997</v>
       </c>
       <c r="W87" s="24" t="s">
         <v>44</v>
@@ -10631,11 +10633,11 @@
         <v>81</v>
       </c>
       <c r="Z87" s="14" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="AB87" s="28"/>
       <c r="AC87" s="22" t="s">
-        <v>913</v>
+        <v>909</v>
       </c>
     </row>
     <row r="88" spans="1:33" ht="60" x14ac:dyDescent="0.25">
@@ -10741,7 +10743,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="90" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A90" s="17">
         <v>89</v>
       </c>
@@ -10788,7 +10790,7 @@
         <v>652</v>
       </c>
       <c r="V90" s="22" t="s">
-        <v>895</v>
+        <v>996</v>
       </c>
       <c r="W90" s="16" t="s">
         <v>44</v>
@@ -10800,16 +10802,16 @@
         <v>92</v>
       </c>
       <c r="Z90" s="14" t="s">
-        <v>990</v>
+        <v>653</v>
       </c>
       <c r="AA90" s="18" t="s">
         <v>704</v>
       </c>
       <c r="AC90" s="22" t="s">
-        <v>989</v>
+        <v>974</v>
       </c>
     </row>
-    <row r="91" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A91" s="17">
         <v>90</v>
       </c>
@@ -10835,16 +10837,16 @@
         <v>628</v>
       </c>
       <c r="M91" s="22" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="N91" s="22" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
       <c r="T91" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V91" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W91" s="24" t="s">
         <v>44</v>
@@ -10856,10 +10858,10 @@
         <v>81</v>
       </c>
       <c r="Z91" s="14" t="s">
-        <v>951</v>
+        <v>980</v>
       </c>
     </row>
-    <row r="92" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A92" s="17">
         <v>91</v>
       </c>
@@ -10885,16 +10887,16 @@
         <v>628</v>
       </c>
       <c r="M92" s="22" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="N92" s="22" t="s">
-        <v>929</v>
+        <v>924</v>
       </c>
       <c r="T92" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V92" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W92" s="24" t="s">
         <v>44</v>
@@ -10906,10 +10908,10 @@
         <v>81</v>
       </c>
       <c r="Z92" s="14" t="s">
-        <v>952</v>
+        <v>981</v>
       </c>
     </row>
-    <row r="93" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A93" s="17">
         <v>92</v>
       </c>
@@ -10935,16 +10937,16 @@
         <v>628</v>
       </c>
       <c r="M93" s="22" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="N93" s="22" t="s">
-        <v>930</v>
+        <v>925</v>
       </c>
       <c r="T93" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V93" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W93" s="24" t="s">
         <v>44</v>
@@ -10956,10 +10958,10 @@
         <v>81</v>
       </c>
       <c r="Z93" s="14" t="s">
-        <v>953</v>
+        <v>982</v>
       </c>
     </row>
-    <row r="94" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A94" s="17">
         <v>93</v>
       </c>
@@ -10985,16 +10987,16 @@
         <v>628</v>
       </c>
       <c r="M94" s="22" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="N94" s="22" t="s">
-        <v>931</v>
+        <v>926</v>
       </c>
       <c r="T94" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V94" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W94" s="24" t="s">
         <v>44</v>
@@ -11006,7 +11008,7 @@
         <v>81</v>
       </c>
       <c r="Z94" s="14" t="s">
-        <v>954</v>
+        <v>983</v>
       </c>
     </row>
     <row r="95" spans="1:33" ht="45" x14ac:dyDescent="0.25">
@@ -11050,7 +11052,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="96" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:33" ht="90" x14ac:dyDescent="0.25">
       <c r="A96" s="17">
         <v>95</v>
       </c>
@@ -11076,16 +11078,16 @@
         <v>628</v>
       </c>
       <c r="M96" s="22" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
       <c r="N96" s="22" t="s">
-        <v>932</v>
+        <v>927</v>
       </c>
       <c r="T96" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V96" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W96" s="24" t="s">
         <v>44</v>
@@ -11097,10 +11099,10 @@
         <v>81</v>
       </c>
       <c r="Z96" s="14" t="s">
-        <v>955</v>
+        <v>984</v>
       </c>
     </row>
-    <row r="97" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A97" s="17">
         <v>96</v>
       </c>
@@ -11126,16 +11128,16 @@
         <v>628</v>
       </c>
       <c r="M97" s="22" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="N97" s="22" t="s">
-        <v>933</v>
+        <v>928</v>
       </c>
       <c r="T97" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V97" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W97" s="24" t="s">
         <v>44</v>
@@ -11147,10 +11149,10 @@
         <v>81</v>
       </c>
       <c r="Z97" s="14" t="s">
-        <v>956</v>
+        <v>985</v>
       </c>
     </row>
-    <row r="98" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A98" s="17">
         <v>97</v>
       </c>
@@ -11176,16 +11178,16 @@
         <v>628</v>
       </c>
       <c r="M98" s="22" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="N98" s="22" t="s">
-        <v>934</v>
+        <v>929</v>
       </c>
       <c r="T98" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V98" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W98" s="24" t="s">
         <v>44</v>
@@ -11197,7 +11199,7 @@
         <v>81</v>
       </c>
       <c r="Z98" s="14" t="s">
-        <v>957</v>
+        <v>986</v>
       </c>
     </row>
     <row r="99" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11226,16 +11228,16 @@
         <v>628</v>
       </c>
       <c r="M99" s="22" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="N99" s="22" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
       <c r="T99" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V99" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W99" s="24" t="s">
         <v>44</v>
@@ -11247,10 +11249,10 @@
         <v>81</v>
       </c>
       <c r="Z99" s="14" t="s">
-        <v>958</v>
+        <v>987</v>
       </c>
     </row>
-    <row r="100" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A100" s="17">
         <v>99</v>
       </c>
@@ -11276,16 +11278,16 @@
         <v>628</v>
       </c>
       <c r="M100" s="22" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="N100" s="22" t="s">
-        <v>936</v>
+        <v>931</v>
       </c>
       <c r="T100" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V100" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W100" s="24" t="s">
         <v>44</v>
@@ -11297,10 +11299,10 @@
         <v>81</v>
       </c>
       <c r="Z100" s="14" t="s">
-        <v>959</v>
+        <v>988</v>
       </c>
     </row>
-    <row r="101" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A101" s="17">
         <v>100</v>
       </c>
@@ -11326,16 +11328,16 @@
         <v>628</v>
       </c>
       <c r="M101" s="22" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="N101" s="22" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="T101" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V101" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W101" s="24" t="s">
         <v>44</v>
@@ -11347,10 +11349,10 @@
         <v>81</v>
       </c>
       <c r="Z101" s="14" t="s">
-        <v>960</v>
+        <v>989</v>
       </c>
     </row>
-    <row r="102" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A102" s="17">
         <v>101</v>
       </c>
@@ -11376,16 +11378,16 @@
         <v>628</v>
       </c>
       <c r="M102" s="22" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
       <c r="N102" s="22" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="T102" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V102" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W102" s="24" t="s">
         <v>44</v>
@@ -11397,10 +11399,10 @@
         <v>81</v>
       </c>
       <c r="Z102" s="14" t="s">
-        <v>961</v>
+        <v>990</v>
       </c>
     </row>
-    <row r="103" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A103" s="17">
         <v>102</v>
       </c>
@@ -11426,16 +11428,16 @@
         <v>628</v>
       </c>
       <c r="M103" s="22" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
       <c r="N103" s="22" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="T103" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V103" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W103" s="24" t="s">
         <v>44</v>
@@ -11447,10 +11449,10 @@
         <v>81</v>
       </c>
       <c r="Z103" s="14" t="s">
-        <v>962</v>
+        <v>991</v>
       </c>
     </row>
-    <row r="104" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A104" s="17">
         <v>103</v>
       </c>
@@ -11476,16 +11478,16 @@
         <v>628</v>
       </c>
       <c r="M104" s="22" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="N104" s="22" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
       <c r="T104" s="22" t="s">
         <v>820</v>
       </c>
       <c r="V104" s="22" t="s">
-        <v>950</v>
+        <v>998</v>
       </c>
       <c r="W104" s="24" t="s">
         <v>44</v>
@@ -11497,7 +11499,7 @@
         <v>81</v>
       </c>
       <c r="Z104" s="14" t="s">
-        <v>963</v>
+        <v>992</v>
       </c>
     </row>
     <row r="105" spans="1:26" ht="45" x14ac:dyDescent="0.25">
@@ -11854,10 +11856,10 @@
         <v>628</v>
       </c>
       <c r="M113" s="22" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
       <c r="N113" s="22" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
       <c r="O113" s="24"/>
       <c r="P113" s="24"/>
@@ -11865,10 +11867,10 @@
       <c r="R113" s="24"/>
       <c r="S113" s="24"/>
       <c r="T113" s="22" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="V113" s="22" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="W113" s="16" t="s">
         <v>44</v>
@@ -11880,7 +11882,7 @@
         <v>81</v>
       </c>
       <c r="Z113" s="14" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="AA113" s="18" t="s">
         <v>777</v>
@@ -11889,7 +11891,7 @@
         <v>778</v>
       </c>
       <c r="AC113" s="22" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
     </row>
     <row r="114" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
@@ -11918,10 +11920,10 @@
         <v>628</v>
       </c>
       <c r="M114" s="22" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
       <c r="N114" s="22" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
       <c r="O114" s="24"/>
       <c r="P114" s="24"/>
@@ -11929,10 +11931,10 @@
       <c r="R114" s="24"/>
       <c r="S114" s="24"/>
       <c r="T114" s="22" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="V114" s="22" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="W114" s="16" t="s">
         <v>44</v>
@@ -11944,13 +11946,13 @@
         <v>81</v>
       </c>
       <c r="Z114" s="14" t="s">
-        <v>948</v>
+        <v>943</v>
       </c>
       <c r="AA114" s="18" t="s">
         <v>782</v>
       </c>
       <c r="AC114" s="22" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
     </row>
     <row r="115" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
@@ -11979,10 +11981,10 @@
         <v>628</v>
       </c>
       <c r="M115" s="22" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
       <c r="N115" s="22" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
       <c r="O115" s="24"/>
       <c r="P115" s="24"/>
@@ -11990,10 +11992,10 @@
       <c r="R115" s="24"/>
       <c r="S115" s="24"/>
       <c r="T115" s="22" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="V115" s="22" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="W115" s="16" t="s">
         <v>44</v>
@@ -12005,7 +12007,7 @@
         <v>81</v>
       </c>
       <c r="Z115" s="14" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
       <c r="AA115" s="18" t="s">
         <v>785</v>
@@ -12014,7 +12016,7 @@
         <v>786</v>
       </c>
       <c r="AC115" s="22" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
     </row>
     <row r="116" spans="1:29" x14ac:dyDescent="0.25">
@@ -12146,7 +12148,7 @@
         <v>81</v>
       </c>
       <c r="Z118" s="14" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
       <c r="AC118" s="22" t="s">
         <v>859</v>

</xml_diff>

<commit_message>
Fixes for energy and CVD ever
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-BCS.xlsx
+++ b/baseline/data_processing_elements-BCS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4CE1C12-BE95-46B3-9DCA-6234A9CF88E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480A0186-A116-4638-B809-5EDADB665E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2109" uniqueCount="999">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="1001">
   <si>
     <t>index</t>
   </si>
@@ -3649,12 +3649,6 @@
     <t>Is the variable B10CHOUR1 'Usual weekly working hours' the correct one to use here? Another variable B10CJSEHS with same label but distribution doesn't look right.</t>
   </si>
   <si>
-    <t>B10ODQENGY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculated Energy (kJ) in diet (excluding supplements)  </t>
-  </si>
-  <si>
     <t>B10DRKFQ</t>
   </si>
   <si>
@@ -3926,12 +3920,6 @@
 ELSE ~ NA_real_)</t>
   </si>
   <si>
-    <t>The study-specific variable is a derived variable calculated based on participant responses about everything they ate and drank in the 24-hour period prior to the day of completion.</t>
-  </si>
-  <si>
-    <t>B10ODQENGY * 0.2390057361</t>
-  </si>
-  <si>
     <t>Use the variable B10ODQENGY from the dietary qx. Harmo comment based on documentation. 
 There are outlier values (0 - &gt;16000).</t>
   </si>
@@ -4008,12 +3996,6 @@
   </si>
   <si>
     <t>There is an option for None of the above. Coded Presumed no based on this.</t>
-  </si>
-  <si>
-    <t>case_when(
-B10KHPB10 == 1 | B10KHPB11 == 1 | B10KHPB20 == 1 ~ 1L; 
-B10KHPB21 == 1 ~ 2L ;
-ELSE ~ NA_integer_)</t>
   </si>
   <si>
     <t>case_when(
@@ -4732,10 +4714,6 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>The study-specific variables ask about types of health problems since last interview/4 years.
-The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
-  </si>
-  <si>
     <t>The study-specific variable asks about types of heart problems since last interview/4 years.
 The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
   </si>
@@ -4755,6 +4733,34 @@
   <si>
     <t>The study-specific variable asks about types of cancer since last interview/4 years.
 The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
+  </si>
+  <si>
+    <t>B10ODQENGY_avg</t>
+  </si>
+  <si>
+    <t>B10ODQENGY_avg * 0.2390057361</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Derived from] Calculated Energy (kJ) in diet (excluding supplements)  </t>
+  </si>
+  <si>
+    <t>The input variable was created in preprocessing and was derived from a study-specific variable based on participant responses about everything they ate and drank in the 24-hour period prior to the day of completion. The derived input variable is a per participant average from entries from the year of the baseline interview, where participants said they ate and drank a typical amount.</t>
+  </si>
+  <si>
+    <t>case_when(
+B10KHPB10 == 1 | B10KHPB11 == 1 | B10KHPB20 == 1 ~ 1L; 
+B10KHPB21 %in% c(0,1) ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>The study-specific variables ask about types of health problems since last interview/4 years.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.  Participants were presumed not to have CVD if they did not select high blood pressure, heart problems, or stroke.</t>
+  </si>
+  <si>
+    <t>Corrected pre-processing to removed duplicates.</t>
+  </si>
+  <si>
+    <t>Updated to presume no for anyone that didn't select high blood pressure, heart problems, or stroke. Previous rule was much more conservative.</t>
   </si>
 </sst>
 </file>
@@ -4868,7 +4874,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -4968,6 +4974,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5332,7 +5347,8 @@
     <col min="28" max="28" width="44.28515625" style="18" customWidth="1"/>
     <col min="29" max="29" width="48.5703125" style="18" customWidth="1"/>
     <col min="30" max="30" width="34.85546875" style="18" customWidth="1"/>
-    <col min="31" max="16384" width="9.140625" style="16"/>
+    <col min="31" max="31" width="24.140625" style="18" customWidth="1"/>
+    <col min="32" max="16384" width="9.140625" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -5571,7 +5587,7 @@
         <v>59</v>
       </c>
       <c r="AC4" s="22" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -5665,7 +5681,7 @@
         <v>78</v>
       </c>
       <c r="V6" s="22" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="W6" s="16" t="s">
         <v>44</v>
@@ -5789,13 +5805,13 @@
         <v>45</v>
       </c>
       <c r="Y8" s="24" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="Z8" s="24" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="AC8" s="18" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
     </row>
     <row r="9" spans="1:33" ht="180" x14ac:dyDescent="0.25">
@@ -5848,7 +5864,7 @@
         <v>116</v>
       </c>
       <c r="V9" s="22" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="W9" s="16" t="s">
         <v>44</v>
@@ -5860,19 +5876,19 @@
         <v>92</v>
       </c>
       <c r="Z9" s="14" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="AA9" s="18" t="s">
         <v>117</v>
       </c>
       <c r="AB9" s="23" t="s">
+        <v>828</v>
+      </c>
+      <c r="AC9" s="22" t="s">
         <v>830</v>
       </c>
-      <c r="AC9" s="22" t="s">
-        <v>832</v>
-      </c>
       <c r="AD9" s="23" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
     </row>
     <row r="10" spans="1:33" ht="165" x14ac:dyDescent="0.25">
@@ -5937,13 +5953,13 @@
         <v>122</v>
       </c>
       <c r="AB10" s="23" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="AC10" s="22" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="AD10" s="23" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
     </row>
     <row r="11" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -5999,7 +6015,7 @@
         <v>134</v>
       </c>
       <c r="V11" s="22" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="W11" s="16" t="s">
         <v>44</v>
@@ -6067,7 +6083,7 @@
         <v>134</v>
       </c>
       <c r="V12" s="22" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="W12" s="16" t="s">
         <v>44</v>
@@ -6135,7 +6151,7 @@
         <v>134</v>
       </c>
       <c r="V13" s="22" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="W13" s="16" t="s">
         <v>147</v>
@@ -6203,7 +6219,7 @@
         <v>134</v>
       </c>
       <c r="V14" s="22" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="W14" s="16" t="s">
         <v>44</v>
@@ -6221,7 +6237,7 @@
         <v>155</v>
       </c>
       <c r="AC14" s="18" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -6277,7 +6293,7 @@
         <v>134</v>
       </c>
       <c r="V15" s="22" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="W15" s="16" t="s">
         <v>44</v>
@@ -6289,10 +6305,10 @@
         <v>92</v>
       </c>
       <c r="Z15" s="14" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="AC15" s="22" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
     </row>
     <row r="16" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -6348,7 +6364,7 @@
         <v>134</v>
       </c>
       <c r="V16" s="22" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="W16" s="16" t="s">
         <v>44</v>
@@ -6360,10 +6376,10 @@
         <v>92</v>
       </c>
       <c r="Z16" s="14" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="AC16" s="22" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
     </row>
     <row r="17" spans="1:30" ht="255" x14ac:dyDescent="0.25">
@@ -6419,7 +6435,7 @@
         <v>134</v>
       </c>
       <c r="V17" s="22" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="W17" s="16" t="s">
         <v>147</v>
@@ -6487,7 +6503,7 @@
         <v>134</v>
       </c>
       <c r="V18" s="22" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="W18" s="16" t="s">
         <v>147</v>
@@ -6555,7 +6571,7 @@
         <v>134</v>
       </c>
       <c r="V19" s="22" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
       <c r="W19" s="16" t="s">
         <v>44</v>
@@ -6620,7 +6636,7 @@
         <v>194</v>
       </c>
       <c r="V20" s="22" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="W20" s="25" t="s">
         <v>44</v>
@@ -6637,7 +6653,7 @@
       <c r="AA20" s="26"/>
       <c r="AB20" s="26"/>
       <c r="AC20" s="22" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
     </row>
     <row r="21" spans="1:30" ht="195" x14ac:dyDescent="0.25">
@@ -6690,7 +6706,7 @@
         <v>194</v>
       </c>
       <c r="V21" s="22" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="W21" s="16" t="s">
         <v>44</v>
@@ -6728,13 +6744,13 @@
         <v>206</v>
       </c>
       <c r="M22" s="18" t="s">
+        <v>847</v>
+      </c>
+      <c r="N22" s="18" t="s">
+        <v>848</v>
+      </c>
+      <c r="T22" s="22" t="s">
         <v>849</v>
-      </c>
-      <c r="N22" s="18" t="s">
-        <v>850</v>
-      </c>
-      <c r="T22" s="22" t="s">
-        <v>851</v>
       </c>
       <c r="W22" s="24" t="s">
         <v>44</v>
@@ -6746,13 +6762,13 @@
         <v>81</v>
       </c>
       <c r="Z22" s="22" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="AB22" s="22" t="s">
         <v>813</v>
       </c>
       <c r="AD22" s="22" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
     </row>
     <row r="23" spans="1:30" ht="255" x14ac:dyDescent="0.25">
@@ -6911,7 +6927,7 @@
         <v>232</v>
       </c>
       <c r="V25" s="22" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="W25" s="16" t="s">
         <v>44</v>
@@ -6926,10 +6942,10 @@
         <v>233</v>
       </c>
       <c r="AA25" s="18" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="AC25" s="22" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
     </row>
     <row r="26" spans="1:30" ht="180" x14ac:dyDescent="0.25">
@@ -6985,7 +7001,7 @@
         <v>246</v>
       </c>
       <c r="V26" s="22" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="W26" s="16" t="s">
         <v>44</v>
@@ -7000,7 +7016,7 @@
         <v>247</v>
       </c>
       <c r="AA26" s="18" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
     </row>
     <row r="27" spans="1:30" ht="135" x14ac:dyDescent="0.25">
@@ -7059,7 +7075,7 @@
         <v>262</v>
       </c>
       <c r="V27" s="22" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="W27" s="16" t="s">
         <v>44</v>
@@ -7189,7 +7205,7 @@
         <v>278</v>
       </c>
       <c r="V29" s="22" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="W29" s="16" t="s">
         <v>44</v>
@@ -7313,7 +7329,7 @@
         <v>292</v>
       </c>
       <c r="V31" s="22" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="W31" s="16" t="s">
         <v>44</v>
@@ -7378,7 +7394,7 @@
         <v>251</v>
       </c>
       <c r="V32" s="22" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="W32" s="16" t="s">
         <v>44</v>
@@ -7390,10 +7406,10 @@
         <v>81</v>
       </c>
       <c r="Z32" s="14" t="s">
-        <v>973</v>
+        <v>968</v>
       </c>
       <c r="AC32" s="22" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
     </row>
     <row r="33" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -7449,10 +7465,10 @@
         <v>81</v>
       </c>
       <c r="Z33" s="14" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="AC33" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="34" spans="1:30" ht="60" x14ac:dyDescent="0.25">
@@ -7508,13 +7524,13 @@
         <v>81</v>
       </c>
       <c r="Z34" s="14" t="s">
-        <v>971</v>
+        <v>966</v>
       </c>
       <c r="AA34" s="18" t="s">
         <v>315</v>
       </c>
       <c r="AC34" s="22" t="s">
-        <v>972</v>
+        <v>967</v>
       </c>
     </row>
     <row r="35" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -7567,10 +7583,10 @@
         <v>81</v>
       </c>
       <c r="Z35" s="14" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="AC35" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="36" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7629,7 +7645,7 @@
         <v>331</v>
       </c>
       <c r="V36" s="22" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="W36" s="16" t="s">
         <v>44</v>
@@ -7638,13 +7654,13 @@
         <v>80</v>
       </c>
       <c r="Y36" s="24" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="Z36" s="20" t="s">
         <v>332</v>
       </c>
       <c r="AC36" s="22" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="37" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7700,7 +7716,7 @@
         <v>331</v>
       </c>
       <c r="V37" s="22" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="W37" s="16" t="s">
         <v>44</v>
@@ -7709,13 +7725,13 @@
         <v>80</v>
       </c>
       <c r="Y37" s="24" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="Z37" s="20" t="s">
         <v>340</v>
       </c>
       <c r="AC37" s="22" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="38" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7771,7 +7787,7 @@
         <v>351</v>
       </c>
       <c r="V38" s="22" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="W38" s="16" t="s">
         <v>44</v>
@@ -7780,13 +7796,13 @@
         <v>80</v>
       </c>
       <c r="Y38" s="24" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="Z38" s="20" t="s">
         <v>352</v>
       </c>
       <c r="AC38" s="22" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="39" spans="1:30" x14ac:dyDescent="0.25">
@@ -7862,7 +7878,7 @@
         <v>51</v>
       </c>
       <c r="V40" s="22" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="W40" s="16" t="s">
         <v>44</v>
@@ -7886,7 +7902,7 @@
         <v>365</v>
       </c>
       <c r="AD40" s="22" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
     </row>
     <row r="41" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -7942,13 +7958,13 @@
         <v>81</v>
       </c>
       <c r="Z41" s="14" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="AA41" s="18" t="s">
         <v>375</v>
       </c>
       <c r="AC41" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="42" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8004,10 +8020,10 @@
         <v>81</v>
       </c>
       <c r="Z42" s="14" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="AC42" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="43" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8063,10 +8079,10 @@
         <v>81</v>
       </c>
       <c r="Z43" s="14" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="AC43" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="44" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8122,10 +8138,10 @@
         <v>81</v>
       </c>
       <c r="Z44" s="14" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="AC44" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="45" spans="1:30" x14ac:dyDescent="0.25">
@@ -8231,13 +8247,13 @@
         <v>81</v>
       </c>
       <c r="Z46" s="14" t="s">
-        <v>967</v>
+        <v>962</v>
       </c>
       <c r="AA46" s="18" t="s">
         <v>409</v>
       </c>
       <c r="AC46" s="22" t="s">
-        <v>966</v>
+        <v>961</v>
       </c>
     </row>
     <row r="47" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8293,10 +8309,10 @@
         <v>81</v>
       </c>
       <c r="Z47" s="14" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="AC47" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -8352,10 +8368,10 @@
         <v>81</v>
       </c>
       <c r="Z48" s="14" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="AC48" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="49" spans="1:31" ht="30" x14ac:dyDescent="0.25">
@@ -8405,7 +8421,7 @@
         <v>428</v>
       </c>
       <c r="AC49" s="18" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
     </row>
     <row r="50" spans="1:31" ht="45" x14ac:dyDescent="0.25">
@@ -8452,7 +8468,7 @@
         <v>428</v>
       </c>
       <c r="AC50" s="18" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="30" x14ac:dyDescent="0.25">
@@ -8502,7 +8518,7 @@
         <v>428</v>
       </c>
       <c r="AC51" s="18" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="45" x14ac:dyDescent="0.25">
@@ -8552,10 +8568,10 @@
         <v>428</v>
       </c>
       <c r="AC52" s="18" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
     </row>
-    <row r="53" spans="1:31" ht="75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" ht="150" x14ac:dyDescent="0.25">
       <c r="A53" s="17">
         <v>52</v>
       </c>
@@ -8577,14 +8593,14 @@
       <c r="G53" s="7" t="s">
         <v>443</v>
       </c>
-      <c r="M53" s="18" t="s">
-        <v>814</v>
-      </c>
-      <c r="N53" s="18" t="s">
-        <v>815</v>
-      </c>
-      <c r="V53" s="22" t="s">
-        <v>876</v>
+      <c r="M53" s="35" t="s">
+        <v>993</v>
+      </c>
+      <c r="N53" s="35" t="s">
+        <v>995</v>
+      </c>
+      <c r="V53" s="35" t="s">
+        <v>996</v>
       </c>
       <c r="W53" s="24" t="s">
         <v>44</v>
@@ -8596,10 +8612,13 @@
         <v>302</v>
       </c>
       <c r="Z53" s="14" t="s">
-        <v>877</v>
+        <v>994</v>
       </c>
       <c r="AC53" s="22" t="s">
-        <v>878</v>
+        <v>874</v>
+      </c>
+      <c r="AE53" s="35" t="s">
+        <v>999</v>
       </c>
     </row>
     <row r="54" spans="1:31" ht="180" x14ac:dyDescent="0.25">
@@ -8649,7 +8668,7 @@
         <v>453</v>
       </c>
       <c r="V54" s="22" t="s">
-        <v>880</v>
+        <v>876</v>
       </c>
       <c r="W54" s="16" t="s">
         <v>44</v>
@@ -8670,12 +8689,12 @@
         <v>456</v>
       </c>
       <c r="AC54" s="22" t="s">
-        <v>879</v>
+        <v>875</v>
       </c>
       <c r="AD54" s="18" t="s">
         <v>457</v>
       </c>
-      <c r="AE54" s="16" t="s">
+      <c r="AE54" s="18" t="s">
         <v>458</v>
       </c>
     </row>
@@ -8702,19 +8721,19 @@
         <v>461</v>
       </c>
       <c r="M55" s="22" t="s">
+        <v>814</v>
+      </c>
+      <c r="N55" s="22" t="s">
+        <v>815</v>
+      </c>
+      <c r="P55" s="24" t="s">
+        <v>877</v>
+      </c>
+      <c r="T55" s="22" t="s">
         <v>816</v>
       </c>
-      <c r="N55" s="22" t="s">
-        <v>817</v>
-      </c>
-      <c r="P55" s="24" t="s">
-        <v>881</v>
-      </c>
-      <c r="T55" s="22" t="s">
-        <v>818</v>
-      </c>
       <c r="V55" s="27" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
       <c r="W55" s="24" t="s">
         <v>44</v>
@@ -8726,10 +8745,10 @@
         <v>92</v>
       </c>
       <c r="Z55" s="14" t="s">
-        <v>884</v>
+        <v>880</v>
       </c>
       <c r="AC55" s="27" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="120" x14ac:dyDescent="0.25">
@@ -8779,7 +8798,7 @@
         <v>471</v>
       </c>
       <c r="V56" s="22" t="s">
-        <v>883</v>
+        <v>879</v>
       </c>
       <c r="W56" s="16" t="s">
         <v>44</v>
@@ -8838,7 +8857,7 @@
         <v>471</v>
       </c>
       <c r="V57" s="22" t="s">
-        <v>883</v>
+        <v>879</v>
       </c>
       <c r="W57" s="16" t="s">
         <v>44</v>
@@ -8850,7 +8869,7 @@
         <v>92</v>
       </c>
       <c r="Z57" s="14" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="75" x14ac:dyDescent="0.25">
@@ -8900,7 +8919,7 @@
         <v>483</v>
       </c>
       <c r="V58" s="22" t="s">
-        <v>886</v>
+        <v>882</v>
       </c>
       <c r="W58" s="16" t="s">
         <v>44</v>
@@ -8912,13 +8931,13 @@
         <v>81</v>
       </c>
       <c r="Z58" s="22" t="s">
-        <v>948</v>
+        <v>943</v>
       </c>
       <c r="AA58" s="18" t="s">
         <v>455</v>
       </c>
       <c r="AC58" s="18" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
     </row>
     <row r="59" spans="1:31" ht="45" x14ac:dyDescent="0.25">
@@ -8971,7 +8990,7 @@
         <v>81</v>
       </c>
       <c r="Z59" s="20" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="195" x14ac:dyDescent="0.25">
@@ -9060,7 +9079,7 @@
       </c>
       <c r="T61" s="21"/>
       <c r="V61" s="22" t="s">
-        <v>887</v>
+        <v>883</v>
       </c>
       <c r="W61" s="16" t="s">
         <v>147</v>
@@ -9081,10 +9100,10 @@
         <v>504</v>
       </c>
       <c r="AC61" s="22" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="AD61" s="23" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
     </row>
     <row r="62" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
@@ -9131,7 +9150,7 @@
         <v>513</v>
       </c>
       <c r="V62" s="22" t="s">
-        <v>968</v>
+        <v>963</v>
       </c>
       <c r="W62" s="16" t="s">
         <v>44</v>
@@ -9146,7 +9165,7 @@
         <v>514</v>
       </c>
       <c r="AC62" s="22" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
     <row r="63" spans="1:31" ht="135" x14ac:dyDescent="0.25">
@@ -9190,7 +9209,7 @@
         <v>520</v>
       </c>
       <c r="V63" s="22" t="s">
-        <v>888</v>
+        <v>884</v>
       </c>
       <c r="W63" s="16" t="s">
         <v>44</v>
@@ -9246,7 +9265,7 @@
         <v>520</v>
       </c>
       <c r="V64" s="22" t="s">
-        <v>888</v>
+        <v>884</v>
       </c>
       <c r="W64" s="16" t="s">
         <v>44</v>
@@ -9261,7 +9280,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="65" spans="1:30" ht="165" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:31" ht="165" x14ac:dyDescent="0.25">
       <c r="A65" s="17">
         <v>64</v>
       </c>
@@ -9299,7 +9318,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="66" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A66" s="17">
         <v>65</v>
       </c>
@@ -9343,7 +9362,7 @@
         <v>520</v>
       </c>
       <c r="V66" s="22" t="s">
-        <v>969</v>
+        <v>964</v>
       </c>
       <c r="W66" s="16" t="s">
         <v>44</v>
@@ -9358,10 +9377,10 @@
         <v>538</v>
       </c>
       <c r="AC66" s="22" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
-    <row r="67" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A67" s="17">
         <v>66</v>
       </c>
@@ -9405,7 +9424,7 @@
         <v>513</v>
       </c>
       <c r="V67" s="22" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="W67" s="16" t="s">
         <v>44</v>
@@ -9420,10 +9439,10 @@
         <v>546</v>
       </c>
       <c r="AC67" s="22" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
-    <row r="68" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:31" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="17">
         <v>67</v>
       </c>
@@ -9464,13 +9483,13 @@
         <v>147</v>
       </c>
       <c r="AB68" s="22" t="s">
-        <v>889</v>
+        <v>885</v>
       </c>
       <c r="AD68" s="23" t="s">
-        <v>890</v>
+        <v>886</v>
       </c>
     </row>
-    <row r="69" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:31" ht="90" x14ac:dyDescent="0.25">
       <c r="A69" s="17">
         <v>68</v>
       </c>
@@ -9508,13 +9527,13 @@
         <v>147</v>
       </c>
       <c r="AB69" s="22" t="s">
-        <v>889</v>
+        <v>885</v>
       </c>
       <c r="AD69" s="23" t="s">
-        <v>890</v>
+        <v>886</v>
       </c>
     </row>
-    <row r="70" spans="1:30" ht="180" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:31" ht="180" x14ac:dyDescent="0.25">
       <c r="A70" s="17">
         <v>69</v>
       </c>
@@ -9558,7 +9577,7 @@
         <v>562</v>
       </c>
       <c r="V70" s="22" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
       <c r="W70" s="16" t="s">
         <v>44</v>
@@ -9573,10 +9592,10 @@
         <v>563</v>
       </c>
       <c r="AC70" s="22" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
-    <row r="71" spans="1:30" ht="105" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:31" ht="105" x14ac:dyDescent="0.25">
       <c r="A71" s="17">
         <v>70</v>
       </c>
@@ -9632,10 +9651,10 @@
         <v>573</v>
       </c>
       <c r="AC71" s="22" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
-    <row r="72" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A72" s="17">
         <v>71</v>
       </c>
@@ -9682,7 +9701,7 @@
         <v>562</v>
       </c>
       <c r="V72" s="22" t="s">
-        <v>891</v>
+        <v>887</v>
       </c>
       <c r="W72" s="16" t="s">
         <v>44</v>
@@ -9697,10 +9716,10 @@
         <v>581</v>
       </c>
       <c r="AC72" s="22" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
-    <row r="73" spans="1:30" ht="135" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:31" ht="135" x14ac:dyDescent="0.25">
       <c r="A73" s="17">
         <v>72</v>
       </c>
@@ -9744,7 +9763,7 @@
         <v>590</v>
       </c>
       <c r="V73" s="27" t="s">
-        <v>903</v>
+        <v>898</v>
       </c>
       <c r="W73" s="16" t="s">
         <v>44</v>
@@ -9759,10 +9778,10 @@
         <v>591</v>
       </c>
       <c r="AC73" s="27" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
     </row>
-    <row r="74" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A74" s="17">
         <v>73</v>
       </c>
@@ -9809,7 +9828,7 @@
         <v>562</v>
       </c>
       <c r="V74" s="22" t="s">
-        <v>891</v>
+        <v>887</v>
       </c>
       <c r="W74" s="16" t="s">
         <v>44</v>
@@ -9824,10 +9843,10 @@
         <v>598</v>
       </c>
       <c r="AC74" s="22" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
-    <row r="75" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:31" ht="45" x14ac:dyDescent="0.25">
       <c r="A75" s="17">
         <v>74</v>
       </c>
@@ -9850,10 +9869,10 @@
         <v>602</v>
       </c>
       <c r="M75" s="22" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
       <c r="N75" s="22" t="s">
-        <v>952</v>
+        <v>947</v>
       </c>
       <c r="O75" s="24" t="s">
         <v>605</v>
@@ -9867,7 +9886,7 @@
         <v>43</v>
       </c>
       <c r="T75" s="33" t="s">
-        <v>954</v>
+        <v>949</v>
       </c>
       <c r="W75" s="32" t="s">
         <v>44</v>
@@ -9879,16 +9898,16 @@
         <v>81</v>
       </c>
       <c r="Z75" s="14" t="s">
-        <v>955</v>
+        <v>950</v>
       </c>
       <c r="AA75" s="22" t="s">
         <v>608</v>
       </c>
       <c r="AC75" s="22" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
     </row>
-    <row r="76" spans="1:30" ht="225" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:31" ht="225" x14ac:dyDescent="0.25">
       <c r="A76" s="17">
         <v>75</v>
       </c>
@@ -9935,16 +9954,16 @@
         <v>80</v>
       </c>
       <c r="Y76" s="24" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="Z76" s="20" t="s">
         <v>613</v>
       </c>
       <c r="AC76" s="22" t="s">
-        <v>892</v>
+        <v>888</v>
       </c>
     </row>
-    <row r="77" spans="1:30" ht="105" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:31" ht="105" x14ac:dyDescent="0.25">
       <c r="A77" s="17">
         <v>76</v>
       </c>
@@ -10000,7 +10019,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="78" spans="1:30" ht="135" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:31" ht="135" x14ac:dyDescent="0.25">
       <c r="A78" s="17">
         <v>77</v>
       </c>
@@ -10029,10 +10048,10 @@
         <v>628</v>
       </c>
       <c r="M78" s="22" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="N78" s="22" t="s">
-        <v>896</v>
+        <v>892</v>
       </c>
       <c r="O78" s="24" t="s">
         <v>629</v>
@@ -10048,8 +10067,8 @@
       <c r="T78" s="31" t="s">
         <v>631</v>
       </c>
-      <c r="V78" s="22" t="s">
-        <v>993</v>
+      <c r="V78" s="35" t="s">
+        <v>998</v>
       </c>
       <c r="W78" s="16" t="s">
         <v>44</v>
@@ -10060,14 +10079,17 @@
       <c r="Y78" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="Z78" s="14" t="s">
-        <v>899</v>
+      <c r="Z78" s="34" t="s">
+        <v>997</v>
       </c>
       <c r="AC78" s="22" t="s">
-        <v>898</v>
+        <v>894</v>
+      </c>
+      <c r="AE78" s="35" t="s">
+        <v>1000</v>
       </c>
     </row>
-    <row r="79" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:31" ht="90" x14ac:dyDescent="0.25">
       <c r="A79" s="17">
         <v>78</v>
       </c>
@@ -10096,16 +10118,16 @@
         <v>628</v>
       </c>
       <c r="M79" s="22" t="s">
-        <v>961</v>
+        <v>956</v>
       </c>
       <c r="N79" s="22" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
       <c r="T79" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V79" s="22" t="s">
-        <v>994</v>
+        <v>988</v>
       </c>
       <c r="W79" s="24" t="s">
         <v>44</v>
@@ -10117,16 +10139,16 @@
         <v>81</v>
       </c>
       <c r="Z79" s="14" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="AB79" s="22" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="AD79" s="23" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
     </row>
-    <row r="80" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:31" ht="90" x14ac:dyDescent="0.25">
       <c r="A80" s="17">
         <v>79</v>
       </c>
@@ -10155,16 +10177,16 @@
         <v>628</v>
       </c>
       <c r="M80" s="22" t="s">
-        <v>962</v>
+        <v>957</v>
       </c>
       <c r="N80" s="22" t="s">
-        <v>957</v>
+        <v>952</v>
       </c>
       <c r="T80" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V80" s="22" t="s">
-        <v>994</v>
+        <v>988</v>
       </c>
       <c r="W80" s="24" t="s">
         <v>44</v>
@@ -10176,16 +10198,16 @@
         <v>81</v>
       </c>
       <c r="Z80" s="14" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="AB80" s="22" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="AC80" s="22" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="AD80" s="23" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
     </row>
     <row r="81" spans="1:33" ht="135" x14ac:dyDescent="0.25">
@@ -10217,16 +10239,16 @@
         <v>628</v>
       </c>
       <c r="M81" s="22" t="s">
-        <v>963</v>
+        <v>958</v>
       </c>
       <c r="N81" s="22" t="s">
-        <v>960</v>
+        <v>955</v>
       </c>
       <c r="T81" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V81" s="22" t="s">
-        <v>995</v>
+        <v>989</v>
       </c>
       <c r="W81" s="24" t="s">
         <v>44</v>
@@ -10238,16 +10260,16 @@
         <v>81</v>
       </c>
       <c r="Z81" s="14" t="s">
-        <v>977</v>
+        <v>972</v>
       </c>
       <c r="AB81" s="22" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="AC81" s="27" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="AD81" s="23" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
     </row>
     <row r="82" spans="1:33" ht="90" x14ac:dyDescent="0.25">
@@ -10297,7 +10319,7 @@
         <v>652</v>
       </c>
       <c r="V82" s="22" t="s">
-        <v>996</v>
+        <v>990</v>
       </c>
       <c r="W82" s="16" t="s">
         <v>44</v>
@@ -10309,16 +10331,16 @@
         <v>92</v>
       </c>
       <c r="Z82" s="14" t="s">
-        <v>978</v>
+        <v>973</v>
       </c>
       <c r="AB82" s="22" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="AC82" s="22" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="AD82" s="23" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
     </row>
     <row r="83" spans="1:33" ht="90" x14ac:dyDescent="0.25">
@@ -10350,16 +10372,16 @@
         <v>628</v>
       </c>
       <c r="M83" s="22" t="s">
-        <v>964</v>
+        <v>959</v>
       </c>
       <c r="N83" s="22" t="s">
-        <v>958</v>
+        <v>953</v>
       </c>
       <c r="T83" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V83" s="22" t="s">
-        <v>994</v>
+        <v>988</v>
       </c>
       <c r="W83" s="24" t="s">
         <v>44</v>
@@ -10371,16 +10393,16 @@
         <v>81</v>
       </c>
       <c r="Z83" s="14" t="s">
-        <v>979</v>
+        <v>974</v>
       </c>
       <c r="AB83" s="22" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="AC83" s="22" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="AD83" s="23" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
     </row>
     <row r="84" spans="1:33" ht="45" x14ac:dyDescent="0.25">
@@ -10427,13 +10449,13 @@
         <v>147</v>
       </c>
       <c r="AB84" s="22" t="s">
-        <v>893</v>
+        <v>889</v>
       </c>
       <c r="AC84" s="22" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="AD84" s="23" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
     </row>
     <row r="85" spans="1:33" ht="90" x14ac:dyDescent="0.25">
@@ -10486,7 +10508,7 @@
         <v>652</v>
       </c>
       <c r="V85" s="22" t="s">
-        <v>996</v>
+        <v>990</v>
       </c>
       <c r="W85" s="16" t="s">
         <v>44</v>
@@ -10498,10 +10520,10 @@
         <v>92</v>
       </c>
       <c r="Z85" s="14" t="s">
-        <v>978</v>
+        <v>973</v>
       </c>
       <c r="AB85" s="22" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
     </row>
     <row r="86" spans="1:33" ht="375" x14ac:dyDescent="0.25">
@@ -10569,17 +10591,17 @@
         <v>81</v>
       </c>
       <c r="Z86" s="14" t="s">
-        <v>900</v>
+        <v>895</v>
       </c>
       <c r="AA86" s="28" t="s">
         <v>455</v>
       </c>
       <c r="AB86" s="28"/>
       <c r="AC86" s="14" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="AD86" s="28"/>
-      <c r="AE86" s="19"/>
+      <c r="AE86" s="28"/>
       <c r="AF86" s="19"/>
       <c r="AG86" s="19"/>
     </row>
@@ -10612,16 +10634,16 @@
         <v>628</v>
       </c>
       <c r="M87" s="22" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="N87" s="22" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="T87" s="22" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="V87" s="22" t="s">
-        <v>997</v>
+        <v>991</v>
       </c>
       <c r="W87" s="24" t="s">
         <v>44</v>
@@ -10633,11 +10655,11 @@
         <v>81</v>
       </c>
       <c r="Z87" s="14" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="AB87" s="28"/>
       <c r="AC87" s="22" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
     </row>
     <row r="88" spans="1:33" ht="60" x14ac:dyDescent="0.25">
@@ -10790,7 +10812,7 @@
         <v>652</v>
       </c>
       <c r="V90" s="22" t="s">
-        <v>996</v>
+        <v>990</v>
       </c>
       <c r="W90" s="16" t="s">
         <v>44</v>
@@ -10808,7 +10830,7 @@
         <v>704</v>
       </c>
       <c r="AC90" s="22" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
     </row>
     <row r="91" spans="1:33" ht="90" x14ac:dyDescent="0.25">
@@ -10837,16 +10859,16 @@
         <v>628</v>
       </c>
       <c r="M91" s="22" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="N91" s="22" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="T91" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V91" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W91" s="24" t="s">
         <v>44</v>
@@ -10858,7 +10880,7 @@
         <v>81</v>
       </c>
       <c r="Z91" s="14" t="s">
-        <v>980</v>
+        <v>975</v>
       </c>
     </row>
     <row r="92" spans="1:33" ht="90" x14ac:dyDescent="0.25">
@@ -10887,16 +10909,16 @@
         <v>628</v>
       </c>
       <c r="M92" s="22" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="N92" s="22" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="T92" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V92" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W92" s="24" t="s">
         <v>44</v>
@@ -10908,7 +10930,7 @@
         <v>81</v>
       </c>
       <c r="Z92" s="14" t="s">
-        <v>981</v>
+        <v>976</v>
       </c>
     </row>
     <row r="93" spans="1:33" ht="90" x14ac:dyDescent="0.25">
@@ -10937,16 +10959,16 @@
         <v>628</v>
       </c>
       <c r="M93" s="22" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="N93" s="22" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
       <c r="T93" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V93" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W93" s="24" t="s">
         <v>44</v>
@@ -10958,7 +10980,7 @@
         <v>81</v>
       </c>
       <c r="Z93" s="14" t="s">
-        <v>982</v>
+        <v>977</v>
       </c>
     </row>
     <row r="94" spans="1:33" ht="90" x14ac:dyDescent="0.25">
@@ -10987,16 +11009,16 @@
         <v>628</v>
       </c>
       <c r="M94" s="22" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="N94" s="22" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
       <c r="T94" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V94" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W94" s="24" t="s">
         <v>44</v>
@@ -11008,7 +11030,7 @@
         <v>81</v>
       </c>
       <c r="Z94" s="14" t="s">
-        <v>983</v>
+        <v>978</v>
       </c>
     </row>
     <row r="95" spans="1:33" ht="45" x14ac:dyDescent="0.25">
@@ -11078,16 +11100,16 @@
         <v>628</v>
       </c>
       <c r="M96" s="22" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="N96" s="22" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="T96" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V96" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W96" s="24" t="s">
         <v>44</v>
@@ -11099,7 +11121,7 @@
         <v>81</v>
       </c>
       <c r="Z96" s="14" t="s">
-        <v>984</v>
+        <v>979</v>
       </c>
     </row>
     <row r="97" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11128,16 +11150,16 @@
         <v>628</v>
       </c>
       <c r="M97" s="22" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="N97" s="22" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
       <c r="T97" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V97" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W97" s="24" t="s">
         <v>44</v>
@@ -11149,7 +11171,7 @@
         <v>81</v>
       </c>
       <c r="Z97" s="14" t="s">
-        <v>985</v>
+        <v>980</v>
       </c>
     </row>
     <row r="98" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11178,16 +11200,16 @@
         <v>628</v>
       </c>
       <c r="M98" s="22" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="N98" s="22" t="s">
-        <v>929</v>
+        <v>924</v>
       </c>
       <c r="T98" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V98" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W98" s="24" t="s">
         <v>44</v>
@@ -11199,7 +11221,7 @@
         <v>81</v>
       </c>
       <c r="Z98" s="14" t="s">
-        <v>986</v>
+        <v>981</v>
       </c>
     </row>
     <row r="99" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11228,16 +11250,16 @@
         <v>628</v>
       </c>
       <c r="M99" s="22" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="N99" s="22" t="s">
-        <v>930</v>
+        <v>925</v>
       </c>
       <c r="T99" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V99" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W99" s="24" t="s">
         <v>44</v>
@@ -11249,7 +11271,7 @@
         <v>81</v>
       </c>
       <c r="Z99" s="14" t="s">
-        <v>987</v>
+        <v>982</v>
       </c>
     </row>
     <row r="100" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11278,16 +11300,16 @@
         <v>628</v>
       </c>
       <c r="M100" s="22" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="N100" s="22" t="s">
-        <v>931</v>
+        <v>926</v>
       </c>
       <c r="T100" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V100" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W100" s="24" t="s">
         <v>44</v>
@@ -11299,7 +11321,7 @@
         <v>81</v>
       </c>
       <c r="Z100" s="14" t="s">
-        <v>988</v>
+        <v>983</v>
       </c>
     </row>
     <row r="101" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11328,16 +11350,16 @@
         <v>628</v>
       </c>
       <c r="M101" s="22" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
       <c r="N101" s="22" t="s">
-        <v>932</v>
+        <v>927</v>
       </c>
       <c r="T101" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V101" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W101" s="24" t="s">
         <v>44</v>
@@ -11349,7 +11371,7 @@
         <v>81</v>
       </c>
       <c r="Z101" s="14" t="s">
-        <v>989</v>
+        <v>984</v>
       </c>
     </row>
     <row r="102" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11378,16 +11400,16 @@
         <v>628</v>
       </c>
       <c r="M102" s="22" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="N102" s="22" t="s">
-        <v>933</v>
+        <v>928</v>
       </c>
       <c r="T102" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V102" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W102" s="24" t="s">
         <v>44</v>
@@ -11399,7 +11421,7 @@
         <v>81</v>
       </c>
       <c r="Z102" s="14" t="s">
-        <v>990</v>
+        <v>985</v>
       </c>
     </row>
     <row r="103" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11428,16 +11450,16 @@
         <v>628</v>
       </c>
       <c r="M103" s="22" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="N103" s="22" t="s">
-        <v>934</v>
+        <v>929</v>
       </c>
       <c r="T103" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V103" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W103" s="24" t="s">
         <v>44</v>
@@ -11449,7 +11471,7 @@
         <v>81</v>
       </c>
       <c r="Z103" s="14" t="s">
-        <v>991</v>
+        <v>986</v>
       </c>
     </row>
     <row r="104" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11478,16 +11500,16 @@
         <v>628</v>
       </c>
       <c r="M104" s="22" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="N104" s="22" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
       <c r="T104" s="22" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="V104" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="W104" s="24" t="s">
         <v>44</v>
@@ -11499,7 +11521,7 @@
         <v>81</v>
       </c>
       <c r="Z104" s="14" t="s">
-        <v>992</v>
+        <v>987</v>
       </c>
     </row>
     <row r="105" spans="1:26" ht="45" x14ac:dyDescent="0.25">
@@ -11527,7 +11549,7 @@
       <c r="L105" s="12" t="s">
         <v>628</v>
       </c>
-      <c r="M105" s="18" t="s">
+      <c r="M105" s="36" t="s">
         <v>51</v>
       </c>
       <c r="W105" s="16" t="s">
@@ -11856,10 +11878,10 @@
         <v>628</v>
       </c>
       <c r="M113" s="22" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="N113" s="22" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="O113" s="24"/>
       <c r="P113" s="24"/>
@@ -11867,10 +11889,10 @@
       <c r="R113" s="24"/>
       <c r="S113" s="24"/>
       <c r="T113" s="22" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="V113" s="22" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
       <c r="W113" s="16" t="s">
         <v>44</v>
@@ -11882,7 +11904,7 @@
         <v>81</v>
       </c>
       <c r="Z113" s="14" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="AA113" s="18" t="s">
         <v>777</v>
@@ -11891,7 +11913,7 @@
         <v>778</v>
       </c>
       <c r="AC113" s="22" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
     </row>
     <row r="114" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
@@ -11920,10 +11942,10 @@
         <v>628</v>
       </c>
       <c r="M114" s="22" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="N114" s="22" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="O114" s="24"/>
       <c r="P114" s="24"/>
@@ -11931,10 +11953,10 @@
       <c r="R114" s="24"/>
       <c r="S114" s="24"/>
       <c r="T114" s="22" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="V114" s="22" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
       <c r="W114" s="16" t="s">
         <v>44</v>
@@ -11946,13 +11968,13 @@
         <v>81</v>
       </c>
       <c r="Z114" s="14" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
       <c r="AA114" s="18" t="s">
         <v>782</v>
       </c>
       <c r="AC114" s="22" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
     </row>
     <row r="115" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
@@ -11981,10 +12003,10 @@
         <v>628</v>
       </c>
       <c r="M115" s="22" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="N115" s="22" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="O115" s="24"/>
       <c r="P115" s="24"/>
@@ -11992,10 +12014,10 @@
       <c r="R115" s="24"/>
       <c r="S115" s="24"/>
       <c r="T115" s="22" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="V115" s="22" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
       <c r="W115" s="16" t="s">
         <v>44</v>
@@ -12007,7 +12029,7 @@
         <v>81</v>
       </c>
       <c r="Z115" s="14" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
       <c r="AA115" s="18" t="s">
         <v>785</v>
@@ -12016,7 +12038,7 @@
         <v>786</v>
       </c>
       <c r="AC115" s="22" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
     </row>
     <row r="116" spans="1:29" x14ac:dyDescent="0.25">
@@ -12148,10 +12170,10 @@
         <v>81</v>
       </c>
       <c r="Z118" s="14" t="s">
-        <v>936</v>
+        <v>931</v>
       </c>
       <c r="AC118" s="22" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="119" spans="1:29" x14ac:dyDescent="0.25">

</xml_diff>